<commit_message>
Portada con el nombre del tour de cada artista
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/preguntas.xlsx
+++ b/datos/preguntas.xlsx
@@ -7,7 +7,7 @@
     <sheet name="INSTRUCCIONES" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'PREGUNTAS'!A1:D211</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'PREGUNTAS'!A1:D210</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D211"/>
+  <dimension ref="A1:D210"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2265,10 +2265,10 @@
         <v>DISCO</v>
       </c>
       <c r="C133" t="str">
-        <v>Real hasta la ___</v>
+        <v>Las leyendas nunca ___</v>
       </c>
       <c r="D133" t="str">
-        <v>MUERTE</v>
+        <v>MUEREN</v>
       </c>
     </row>
     <row r="134">
@@ -2276,13 +2276,13 @@
         <v>ANUEL AA</v>
       </c>
       <c r="B134" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C134" t="str">
-        <v>Las leyendas nunca ___</v>
+        <v>Su disco con Ozuna se llama Los ___</v>
       </c>
       <c r="D134" t="str">
-        <v>MUEREN</v>
+        <v>DIOSES</v>
       </c>
     </row>
     <row r="135">
@@ -2293,10 +2293,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C135" t="str">
-        <v>Su disco con Ozuna se llama Los ___</v>
+        <v>¿Cómo se llama su disco de 2020, que lleva su primer nombre?</v>
       </c>
       <c r="D135" t="str">
-        <v>DIOSES</v>
+        <v>EMMANUEL</v>
       </c>
     </row>
     <row r="136">
@@ -2307,10 +2307,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C136" t="str">
-        <v>¿Cómo se llama su disco de 2020, que lleva su primer nombre?</v>
+        <v>Su nombre real es Emmanuel ___ Santiago</v>
       </c>
       <c r="D136" t="str">
-        <v>EMMANUEL</v>
+        <v>GAZMEY</v>
       </c>
     </row>
     <row r="137">
@@ -2321,10 +2321,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C137" t="str">
-        <v>Su nombre real es Emmanuel ___ Santiago</v>
+        <v>Anuel AA nació en Carolina, Puerto ___</v>
       </c>
       <c r="D137" t="str">
-        <v>GAZMEY</v>
+        <v>RICO</v>
       </c>
     </row>
     <row r="138">
@@ -2335,10 +2335,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C138" t="str">
-        <v>Anuel AA nació en Carolina, Puerto ___</v>
+        <v>¿Con qué cantante puertorriqueño grabó el disco «Los Dioses»?</v>
       </c>
       <c r="D138" t="str">
-        <v>RICO</v>
+        <v>OZUNA</v>
       </c>
     </row>
     <row r="139">
@@ -2349,10 +2349,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C139" t="str">
-        <v>¿Con qué cantante puertorriqueño grabó el disco «Los Dioses»?</v>
+        <v>¿Qué canción de 2019 grabó con Karol G?</v>
       </c>
       <c r="D139" t="str">
-        <v>OZUNA</v>
+        <v>SECRETO</v>
       </c>
     </row>
     <row r="140">
@@ -2363,10 +2363,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C140" t="str">
-        <v>¿Qué canción de 2019 grabó con Karol G?</v>
+        <v>¿Qué canción de 2019 junta a Anuel con Daddy Yankee, Karol G, Ozuna y J Balvin?</v>
       </c>
       <c r="D140" t="str">
-        <v>SECRETO</v>
+        <v>CHINA</v>
       </c>
     </row>
     <row r="141">
@@ -2377,10 +2377,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C141" t="str">
-        <v>¿Qué canción de 2019 junta a Anuel con Daddy Yankee, Karol G, Ozuna y J Balvin?</v>
+        <v>¿Qué canción grabó con Tekashi 6ix9ine en 2018?</v>
       </c>
       <c r="D141" t="str">
-        <v>CHINA</v>
+        <v>BEBÉ</v>
       </c>
     </row>
     <row r="142">
@@ -2391,10 +2391,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C142" t="str">
-        <v>¿Qué canción grabó con Tekashi 6ix9ine en 2018?</v>
+        <v>¿Cómo se llama su primer gran éxito, de 2016?</v>
       </c>
       <c r="D142" t="str">
-        <v>BEBÉ</v>
+        <v>SOLA</v>
       </c>
     </row>
     <row r="143">
@@ -2405,10 +2405,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C143" t="str">
-        <v>¿Cómo se llama su primer gran éxito, de 2016?</v>
+        <v>El remix de «Sola» lo grabó con Daddy Yankee, Wisin, Farruko y Zion &amp; ___</v>
       </c>
       <c r="D143" t="str">
-        <v>SOLA</v>
+        <v>LENNOX</v>
       </c>
     </row>
     <row r="144">
@@ -2419,10 +2419,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C144" t="str">
-        <v>El remix de «Sola» lo grabó con Daddy Yankee, Wisin, Farruko y Zion &amp; ___</v>
+        <v>«Adicto» la grabó con Ozuna y el productor ___</v>
       </c>
       <c r="D144" t="str">
-        <v>LENNOX</v>
+        <v>TAINY</v>
       </c>
     </row>
     <row r="145">
@@ -2433,10 +2433,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C145" t="str">
-        <v>«Adicto» la grabó con Ozuna y el productor ___</v>
+        <v>«Hasta que Dios diga» la grabó con Bad ___</v>
       </c>
       <c r="D145" t="str">
-        <v>TAINY</v>
+        <v>BUNNY</v>
       </c>
     </row>
     <row r="146">
@@ -2447,24 +2447,24 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C146" t="str">
-        <v>«Hasta que Dios diga» la grabó con Bad ___</v>
+        <v>Además del reguetón, su género es el ___ latino</v>
       </c>
       <c r="D146" t="str">
-        <v>BUNNY</v>
+        <v>TRAP</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B147" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C147" t="str">
-        <v>Además del reguetón, su género es el ___ latino</v>
+        <v>¿Cómo se llama el estadio de Tigres? Estadio ___</v>
       </c>
       <c r="D147" t="str">
-        <v>TRAP</v>
+        <v>UNIVERSITARIO</v>
       </c>
     </row>
     <row r="148">
@@ -2475,10 +2475,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C148" t="str">
-        <v>¿Cómo se llama el estadio de Tigres? Estadio ___</v>
+        <v>¿Cómo le dicen al Estadio Universitario por lo caliente de su ambiente?</v>
       </c>
       <c r="D148" t="str">
-        <v>UNIVERSITARIO</v>
+        <v>VOLCÁN</v>
       </c>
     </row>
     <row r="149">
@@ -2489,10 +2489,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C149" t="str">
-        <v>¿Cómo le dicen al Estadio Universitario por lo caliente de su ambiente?</v>
+        <v>El Volcán está en el municipio de San Nicolás de los ___</v>
       </c>
       <c r="D149" t="str">
-        <v>VOLCÁN</v>
+        <v>GARZA</v>
       </c>
     </row>
     <row r="150">
@@ -2503,10 +2503,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C150" t="str">
-        <v>El Volcán está en el municipio de San Nicolás de los ___</v>
+        <v>Tigres es el equipo de la Universidad Autónoma de Nuevo ___</v>
       </c>
       <c r="D150" t="str">
-        <v>GARZA</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="151">
@@ -2517,10 +2517,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C151" t="str">
-        <v>Tigres es el equipo de la Universidad Autónoma de Nuevo ___</v>
+        <v>¿En qué año se fundó Tigres?</v>
       </c>
       <c r="D151" t="str">
-        <v>LEÓN</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="152">
@@ -2531,10 +2531,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C152" t="str">
-        <v>¿En qué año se fundó Tigres?</v>
+        <v>Los colores de Tigres son el azul y el ___</v>
       </c>
       <c r="D152" t="str">
-        <v>1960</v>
+        <v>AMARILLO</v>
       </c>
     </row>
     <row r="153">
@@ -2545,10 +2545,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C153" t="str">
-        <v>Los colores de Tigres son el azul y el ___</v>
+        <v>Por su uniforme amarillo y azul, a Tigres también le dicen los ___</v>
       </c>
       <c r="D153" t="str">
-        <v>AMARILLO</v>
+        <v>AURIAZULES</v>
       </c>
     </row>
     <row r="154">
@@ -2559,10 +2559,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C154" t="str">
-        <v>Por su uniforme amarillo y azul, a Tigres también le dicen los ___</v>
+        <v>¿Qué animal es el emblema de la UANL?</v>
       </c>
       <c r="D154" t="str">
-        <v>AURIAZULES</v>
+        <v>TIGRE</v>
       </c>
     </row>
     <row r="155">
@@ -2573,10 +2573,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C155" t="str">
-        <v>¿Qué animal es el emblema de la UANL?</v>
+        <v>¿Cómo se apellida André-Pierre, el máximo goleador en la historia de Tigres?</v>
       </c>
       <c r="D155" t="str">
-        <v>TIGRE</v>
+        <v>GIGNAC</v>
       </c>
     </row>
     <row r="156">
@@ -2587,10 +2587,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C156" t="str">
-        <v>¿Cómo se apellida André-Pierre, el máximo goleador en la historia de Tigres?</v>
+        <v>¿De qué país es André-Pierre Gignac?</v>
       </c>
       <c r="D156" t="str">
-        <v>GIGNAC</v>
+        <v>FRANCIA</v>
       </c>
     </row>
     <row r="157">
@@ -2601,10 +2601,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C157" t="str">
-        <v>¿De qué país es André-Pierre Gignac?</v>
+        <v>Con el técnico Ricardo «Tuca» ___, Tigres ganó cinco títulos de liga</v>
       </c>
       <c r="D157" t="str">
-        <v>FRANCIA</v>
+        <v>FERRETTI</v>
       </c>
     </row>
     <row r="158">
@@ -2615,10 +2615,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C158" t="str">
-        <v>Con el técnico Ricardo «Tuca» ___, Tigres ganó cinco títulos de liga</v>
+        <v>¿De qué país es el técnico Ricardo «Tuca» Ferretti?</v>
       </c>
       <c r="D158" t="str">
-        <v>FERRETTI</v>
+        <v>BRASIL</v>
       </c>
     </row>
     <row r="159">
@@ -2629,10 +2629,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C159" t="str">
-        <v>¿De qué país es el técnico Ricardo «Tuca» Ferretti?</v>
+        <v>Al portero argentino Nahuel Guzmán le apodan «El ___»</v>
       </c>
       <c r="D159" t="str">
-        <v>BRASIL</v>
+        <v>PATÓN</v>
       </c>
     </row>
     <row r="160">
@@ -2643,10 +2643,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C160" t="str">
-        <v>Al portero argentino Nahuel Guzmán le apodan «El ___»</v>
+        <v>El mediocampista argentino que fue capitán de Tigres: Guido ___</v>
       </c>
       <c r="D160" t="str">
-        <v>PATÓN</v>
+        <v>PIZARRO</v>
       </c>
     </row>
     <row r="161">
@@ -2657,10 +2657,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C161" t="str">
-        <v>El mediocampista argentino que fue capitán de Tigres: Guido ___</v>
+        <v>En 2020 Tigres ganó la Concacaf ___ League</v>
       </c>
       <c r="D161" t="str">
-        <v>PIZARRO</v>
+        <v>CHAMPIONS</v>
       </c>
     </row>
     <row r="162">
@@ -2671,10 +2671,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C162" t="str">
-        <v>En 2020 Tigres ganó la Concacaf ___ League</v>
+        <v>En la final del Mundial de Clubes 2020, Tigres enfrentó al Bayern ___</v>
       </c>
       <c r="D162" t="str">
-        <v>CHAMPIONS</v>
+        <v>MÚNICH</v>
       </c>
     </row>
     <row r="163">
@@ -2685,10 +2685,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C163" t="str">
-        <v>En la final del Mundial de Clubes 2020, Tigres enfrentó al Bayern ___</v>
+        <v>A la afición de Tigres se le conoce como «La afición ___»</v>
       </c>
       <c r="D163" t="str">
-        <v>MÚNICH</v>
+        <v>INCOMPARABLE</v>
       </c>
     </row>
     <row r="164">
@@ -2699,10 +2699,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C164" t="str">
-        <v>A la afición de Tigres se le conoce como «La afición ___»</v>
+        <v>La barra de Tigres se llama Libres y ___</v>
       </c>
       <c r="D164" t="str">
-        <v>INCOMPARABLE</v>
+        <v>LOKOS</v>
       </c>
     </row>
     <row r="165">
@@ -2713,10 +2713,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C165" t="str">
-        <v>La barra de Tigres se llama Libres y ___</v>
+        <v>El partido entre Tigres y Rayados se llama el Clásico ___</v>
       </c>
       <c r="D165" t="str">
-        <v>LOKOS</v>
+        <v>REGIO</v>
       </c>
     </row>
     <row r="166">
@@ -2727,24 +2727,24 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C166" t="str">
-        <v>El partido entre Tigres y Rayados se llama el Clásico ___</v>
+        <v>¿Cómo se llama el equipo de mujeres de la UANL? Tigres ___</v>
       </c>
       <c r="D166" t="str">
-        <v>REGIO</v>
+        <v>FEMENIL</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B167" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C167" t="str">
-        <v>¿Cómo se llama el equipo de mujeres de la UANL? Tigres ___</v>
+        <v>¿Cómo se llama el estadio de Rayados? Estadio ___</v>
       </c>
       <c r="D167" t="str">
-        <v>FEMENIL</v>
+        <v>BBVA</v>
       </c>
     </row>
     <row r="168">
@@ -2755,10 +2755,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C168" t="str">
-        <v>¿Cómo se llama el estadio de Rayados? Estadio ___</v>
+        <v>Al Estadio BBVA le dicen el Gigante de ___</v>
       </c>
       <c r="D168" t="str">
-        <v>BBVA</v>
+        <v>ACERO</v>
       </c>
     </row>
     <row r="169">
@@ -2769,10 +2769,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C169" t="str">
-        <v>Al Estadio BBVA le dicen el Gigante de ___</v>
+        <v>¿En qué año se inauguró el Estadio BBVA?</v>
       </c>
       <c r="D169" t="str">
-        <v>ACERO</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="170">
@@ -2783,10 +2783,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C170" t="str">
-        <v>¿En qué año se inauguró el Estadio BBVA?</v>
+        <v>¿En qué municipio está el Estadio BBVA?</v>
       </c>
       <c r="D170" t="str">
-        <v>2015</v>
+        <v>GUADALUPE</v>
       </c>
     </row>
     <row r="171">
@@ -2797,10 +2797,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C171" t="str">
-        <v>¿En qué municipio está el Estadio BBVA?</v>
+        <v>El Estadio BBVA está junto al parque ecológico La ___</v>
       </c>
       <c r="D171" t="str">
-        <v>GUADALUPE</v>
+        <v>PASTORA</v>
       </c>
     </row>
     <row r="172">
@@ -2811,10 +2811,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C172" t="str">
-        <v>El Estadio BBVA está junto al parque ecológico La ___</v>
+        <v>Desde las gradas del BBVA se ve el Cerro de la ___</v>
       </c>
       <c r="D172" t="str">
-        <v>PASTORA</v>
+        <v>SILLA</v>
       </c>
     </row>
     <row r="173">
@@ -2825,10 +2825,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C173" t="str">
-        <v>Desde las gradas del BBVA se ve el Cerro de la ___</v>
+        <v>Antes del BBVA, Rayados jugaba de local en el Estadio ___</v>
       </c>
       <c r="D173" t="str">
-        <v>SILLA</v>
+        <v>TECNOLÓGICO</v>
       </c>
     </row>
     <row r="174">
@@ -2839,10 +2839,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C174" t="str">
-        <v>Antes del BBVA, Rayados jugaba de local en el Estadio ___</v>
+        <v>El nombre oficial de Rayados es Club de Futbol ___</v>
       </c>
       <c r="D174" t="str">
-        <v>TECNOLÓGICO</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="175">
@@ -2853,10 +2853,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C175" t="str">
-        <v>El nombre oficial de Rayados es Club de Futbol ___</v>
+        <v>¿En qué año se fundó Rayados?</v>
       </c>
       <c r="D175" t="str">
-        <v>MONTERREY</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="176">
@@ -2867,10 +2867,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C176" t="str">
-        <v>¿En qué año se fundó Rayados?</v>
+        <v>El uniforme de Rayados tiene rayas verticales azules y ___</v>
       </c>
       <c r="D176" t="str">
-        <v>1945</v>
+        <v>BLANCAS</v>
       </c>
     </row>
     <row r="177">
@@ -2881,10 +2881,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C177" t="str">
-        <v>El uniforme de Rayados tiene rayas verticales azules y ___</v>
+        <v>Además de Rayados, al equipo también le dicen La ___</v>
       </c>
       <c r="D177" t="str">
-        <v>BLANCAS</v>
+        <v>PANDILLA</v>
       </c>
     </row>
     <row r="178">
@@ -2895,10 +2895,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C178" t="str">
-        <v>Además de Rayados, al equipo también le dicen La ___</v>
+        <v>¿En qué año ganó Rayados su primer título de liga?</v>
       </c>
       <c r="D178" t="str">
-        <v>PANDILLA</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="179">
@@ -2909,10 +2909,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C179" t="str">
-        <v>¿En qué año ganó Rayados su primer título de liga?</v>
+        <v>Entre 2011 y 2013, ¿cuántas Concachampions seguidas ganó Rayados?</v>
       </c>
       <c r="D179" t="str">
-        <v>1986</v>
+        <v>TRES</v>
       </c>
     </row>
     <row r="180">
@@ -2923,10 +2923,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C180" t="str">
-        <v>Entre 2011 y 2013, ¿cuántas Concachampions seguidas ganó Rayados?</v>
+        <v>Al técnico Víctor Manuel Vucetich le dicen el Rey ___</v>
       </c>
       <c r="D180" t="str">
-        <v>TRES</v>
+        <v>MIDAS</v>
       </c>
     </row>
     <row r="181">
@@ -2937,10 +2937,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C181" t="str">
-        <v>Al técnico Víctor Manuel Vucetich le dicen el Rey ___</v>
+        <v>Al delantero chileno Humberto Suazo le decían «___»</v>
       </c>
       <c r="D181" t="str">
-        <v>MIDAS</v>
+        <v>CHUPETE</v>
       </c>
     </row>
     <row r="182">
@@ -2951,10 +2951,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C182" t="str">
-        <v>Al delantero chileno Humberto Suazo le decían «___»</v>
+        <v>El máximo goleador en la historia de Rayados es Rogelio Funes ___</v>
       </c>
       <c r="D182" t="str">
-        <v>CHUPETE</v>
+        <v>MORI</v>
       </c>
     </row>
     <row r="183">
@@ -2965,10 +2965,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C183" t="str">
-        <v>El máximo goleador en la historia de Rayados es Rogelio Funes ___</v>
+        <v>Al ídolo regiomontano Jesús Arellano le decían «El ___»</v>
       </c>
       <c r="D183" t="str">
-        <v>MORI</v>
+        <v>CABRITO</v>
       </c>
     </row>
     <row r="184">
@@ -2979,10 +2979,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C184" t="str">
-        <v>Al ídolo regiomontano Jesús Arellano le decían «El ___»</v>
+        <v>En 2025 llegó a Rayados el famoso defensa español Sergio ___</v>
       </c>
       <c r="D184" t="str">
-        <v>CABRITO</v>
+        <v>RAMOS</v>
       </c>
     </row>
     <row r="185">
@@ -2993,10 +2993,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C185" t="str">
-        <v>En 2025 llegó a Rayados el famoso defensa español Sergio ___</v>
+        <v>Rayados quedó en tercer lugar del Mundial de ___ en 2012 y en 2019</v>
       </c>
       <c r="D185" t="str">
-        <v>RAMOS</v>
+        <v>CLUBES</v>
       </c>
     </row>
     <row r="186">
@@ -3007,10 +3007,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C186" t="str">
-        <v>Rayados quedó en tercer lugar del Mundial de ___ en 2012 y en 2019</v>
+        <v>A la barra de Rayados se le conoce como La ___</v>
       </c>
       <c r="D186" t="str">
-        <v>CLUBES</v>
+        <v>ADICCIÓN</v>
       </c>
     </row>
     <row r="187">
@@ -3021,10 +3021,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C187" t="str">
-        <v>A la barra de Rayados se le conoce como La ___</v>
+        <v>El partido entre Rayados y Tigres se llama el Clásico ___</v>
       </c>
       <c r="D187" t="str">
-        <v>ADICCIÓN</v>
+        <v>REGIO</v>
       </c>
     </row>
     <row r="188">
@@ -3035,24 +3035,24 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C188" t="str">
-        <v>El partido entre Rayados y Tigres se llama el Clásico ___</v>
+        <v>Monterrey es la capital del estado de Nuevo ___</v>
       </c>
       <c r="D188" t="str">
-        <v>REGIO</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B189" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C189" t="str">
-        <v>Monterrey es la capital del estado de Nuevo ___</v>
+        <v>El equipo del Tec de Monterrey se llama Borregos ___</v>
       </c>
       <c r="D189" t="str">
-        <v>LEÓN</v>
+        <v>SALVAJES</v>
       </c>
     </row>
     <row r="190">
@@ -3063,10 +3063,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C190" t="str">
-        <v>El equipo del Tec de Monterrey se llama Borregos ___</v>
+        <v>Los Borregos juegan futbol ___</v>
       </c>
       <c r="D190" t="str">
-        <v>SALVAJES</v>
+        <v>AMERICANO</v>
       </c>
     </row>
     <row r="191">
@@ -3077,10 +3077,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C191" t="str">
-        <v>Los Borregos juegan futbol ___</v>
+        <v>Borregos es el equipo del Tecnológico de ___</v>
       </c>
       <c r="D191" t="str">
-        <v>AMERICANO</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="192">
@@ -3091,10 +3091,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C192" t="str">
-        <v>Borregos es el equipo del Tecnológico de ___</v>
+        <v>El Tec de Monterrey lo fundó el empresario Eugenio Garza ___</v>
       </c>
       <c r="D192" t="str">
-        <v>MONTERREY</v>
+        <v>SADA</v>
       </c>
     </row>
     <row r="193">
@@ -3105,10 +3105,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C193" t="str">
-        <v>El Tec de Monterrey lo fundó el empresario Eugenio Garza ___</v>
+        <v>¿En qué año se fundó el Tec de Monterrey?</v>
       </c>
       <c r="D193" t="str">
-        <v>SADA</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="194">
@@ -3119,10 +3119,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C194" t="str">
-        <v>¿En qué año se fundó el Tec de Monterrey?</v>
+        <v>Los colores de Borregos son el azul y el ___</v>
       </c>
       <c r="D194" t="str">
-        <v>1943</v>
+        <v>BLANCO</v>
       </c>
     </row>
     <row r="195">
@@ -3133,10 +3133,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C195" t="str">
-        <v>Los colores de Borregos son el azul y el ___</v>
+        <v>¿En qué año se inauguró el Estadio Borregos?</v>
       </c>
       <c r="D195" t="str">
-        <v>BLANCO</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="196">
@@ -3147,10 +3147,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C196" t="str">
-        <v>¿En qué año se inauguró el Estadio Borregos?</v>
+        <v>El Estadio Borregos se construyó en el lugar del antiguo Estadio ___</v>
       </c>
       <c r="D196" t="str">
-        <v>2019</v>
+        <v>TECNOLÓGICO</v>
       </c>
     </row>
     <row r="197">
@@ -3161,10 +3161,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C197" t="str">
-        <v>El Estadio Borregos se construyó en el lugar del antiguo Estadio ___</v>
+        <v>¿Qué equipo de futbol soccer jugó en el Estadio Tecnológico hasta 2015?</v>
       </c>
       <c r="D197" t="str">
-        <v>TECNOLÓGICO</v>
+        <v>RAYADOS</v>
       </c>
     </row>
     <row r="198">
@@ -3175,10 +3175,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C198" t="str">
-        <v>¿Qué equipo de futbol soccer jugó en el Estadio Tecnológico hasta 2015?</v>
+        <v>¿Cómo se llama la liga universitaria de futbol americano donde juega Borregos?</v>
       </c>
       <c r="D198" t="str">
-        <v>RAYADOS</v>
+        <v>ONEFA</v>
       </c>
     </row>
     <row r="199">
@@ -3189,10 +3189,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C199" t="str">
-        <v>¿Cómo se llama la liga universitaria de futbol americano donde juega Borregos?</v>
+        <v>El gran rival universitario de Borregos son los Auténticos ___</v>
       </c>
       <c r="D199" t="str">
-        <v>ONEFA</v>
+        <v>TIGRES</v>
       </c>
     </row>
     <row r="200">
@@ -3203,10 +3203,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C200" t="str">
-        <v>El gran rival universitario de Borregos son los Auténticos ___</v>
+        <v>El legendario coach de Borregos Monterrey fue Frank ___</v>
       </c>
       <c r="D200" t="str">
-        <v>TIGRES</v>
+        <v>GONZÁLEZ</v>
       </c>
     </row>
     <row r="201">
@@ -3217,10 +3217,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C201" t="str">
-        <v>El legendario coach de Borregos Monterrey fue Frank ___</v>
+        <v>¿Qué animal es la mascota del Tec de Monterrey?</v>
       </c>
       <c r="D201" t="str">
-        <v>GONZÁLEZ</v>
+        <v>BORREGO</v>
       </c>
     </row>
     <row r="202">
@@ -3231,10 +3231,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C202" t="str">
-        <v>¿Qué animal es la mascota del Tec de Monterrey?</v>
+        <v>Llevar el balón hasta la zona de anotación es un ___</v>
       </c>
       <c r="D202" t="str">
-        <v>BORREGO</v>
+        <v>TOUCHDOWN</v>
       </c>
     </row>
     <row r="203">
@@ -3245,10 +3245,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C203" t="str">
-        <v>Llevar el balón hasta la zona de anotación es un ___</v>
+        <v>¿Cuántos puntos vale un touchdown?</v>
       </c>
       <c r="D203" t="str">
-        <v>TOUCHDOWN</v>
+        <v>SEIS</v>
       </c>
     </row>
     <row r="204">
@@ -3259,10 +3259,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C204" t="str">
-        <v>¿Cuántos puntos vale un touchdown?</v>
+        <v>¿Cuántos puntos vale un gol de campo?</v>
       </c>
       <c r="D204" t="str">
-        <v>SEIS</v>
+        <v>TRES</v>
       </c>
     </row>
     <row r="205">
@@ -3273,10 +3273,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C205" t="str">
-        <v>¿Cuántos puntos vale un gol de campo?</v>
+        <v>¿Cuántos puntos vale un safety?</v>
       </c>
       <c r="D205" t="str">
-        <v>TRES</v>
+        <v>DOS</v>
       </c>
     </row>
     <row r="206">
@@ -3287,10 +3287,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C206" t="str">
-        <v>¿Cuántos puntos vale un safety?</v>
+        <v>Después de un touchdown se patea para ganar el punto ___</v>
       </c>
       <c r="D206" t="str">
-        <v>DOS</v>
+        <v>EXTRA</v>
       </c>
     </row>
     <row r="207">
@@ -3301,10 +3301,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C207" t="str">
-        <v>Después de un touchdown se patea para ganar el punto ___</v>
+        <v>El jugador que lanza los pases es el mariscal de ___</v>
       </c>
       <c r="D207" t="str">
-        <v>EXTRA</v>
+        <v>CAMPO</v>
       </c>
     </row>
     <row r="208">
@@ -3315,10 +3315,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C208" t="str">
-        <v>El jugador que lanza los pases es el mariscal de ___</v>
+        <v>¿Cuántos jugadores tiene cada equipo en la cancha?</v>
       </c>
       <c r="D208" t="str">
-        <v>CAMPO</v>
+        <v>ONCE</v>
       </c>
     </row>
     <row r="209">
@@ -3329,10 +3329,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C209" t="str">
-        <v>¿Cuántos jugadores tiene cada equipo en la cancha?</v>
+        <v>¿En cuántas oportunidades hay que avanzar diez yardas?</v>
       </c>
       <c r="D209" t="str">
-        <v>ONCE</v>
+        <v>CUATRO</v>
       </c>
     </row>
     <row r="210">
@@ -3343,30 +3343,16 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C210" t="str">
-        <v>¿En cuántas oportunidades hay que avanzar diez yardas?</v>
+        <v>La gran final de la NFL se llama el Super ___</v>
       </c>
       <c r="D210" t="str">
-        <v>CUATRO</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B211" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C211" t="str">
-        <v>La gran final de la NFL se llama el Super ___</v>
-      </c>
-      <c r="D211" t="str">
         <v>BOWL</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D211"/>
+  <autoFilter ref="A1:D210"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D211"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D210"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Sin nombres de artistas en pantalla (derechos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/preguntas.xlsx
+++ b/datos/preguntas.xlsx
@@ -7,7 +7,7 @@
     <sheet name="INSTRUCCIONES" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'PREGUNTAS'!A1:D210</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'PREGUNTAS'!A1:D204</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D210"/>
+  <dimension ref="A1:D204"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -739,10 +739,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C24" t="str">
-        <v>¿Cómo se apellida Adam, el vocalista de Maroon 5?</v>
+        <v>¿Qué instrumento toca el vocalista de la banda además de cantar?</v>
       </c>
       <c r="D24" t="str">
-        <v>LEVINE</v>
+        <v>GUITARRA</v>
       </c>
     </row>
     <row r="25">
@@ -753,10 +753,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C25" t="str">
-        <v>¿Qué instrumento toca Adam Levine además de cantar?</v>
+        <v>Antes de tener su nombre actual, la banda se llamaba Kara's ___</v>
       </c>
       <c r="D25" t="str">
-        <v>GUITARRA</v>
+        <v>FLOWERS</v>
       </c>
     </row>
     <row r="26">
@@ -767,10 +767,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C26" t="str">
-        <v>Antes de llamarse Maroon 5, la banda se llamaba Kara's ___</v>
+        <v>La banda se formó en la ciudad de Los ___, California</v>
       </c>
       <c r="D26" t="str">
-        <v>FLOWERS</v>
+        <v>ÁNGELES</v>
       </c>
     </row>
     <row r="27">
@@ -781,10 +781,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C27" t="str">
-        <v>Maroon 5 se formó en la ciudad de Los ___, California</v>
+        <v>¿Qué canción grabó la banda con Wiz Khalifa?</v>
       </c>
       <c r="D27" t="str">
-        <v>ÁNGELES</v>
+        <v>PAYPHONE</v>
       </c>
     </row>
     <row r="28">
@@ -795,10 +795,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C28" t="str">
-        <v>¿Qué canción de Maroon 5 grabaron con Wiz Khalifa?</v>
+        <v>¿Qué canción grabó la banda con el rapero Future?</v>
       </c>
       <c r="D28" t="str">
-        <v>PAYPHONE</v>
+        <v>COLD</v>
       </c>
     </row>
     <row r="29">
@@ -809,10 +809,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C29" t="str">
-        <v>¿Qué canción de Maroon 5 grabaron con el rapero Future?</v>
+        <v>¿En el video de qué canción la banda llega de sorpresa a varias bodas?</v>
       </c>
       <c r="D29" t="str">
-        <v>COLD</v>
+        <v>SUGAR</v>
       </c>
     </row>
     <row r="30">
@@ -823,10 +823,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C30" t="str">
-        <v>¿En el video de qué canción la banda llega de sorpresa a varias bodas?</v>
+        <v>¿Qué canción de 2019 es un brindis por los seres queridos que ya no están?</v>
       </c>
       <c r="D30" t="str">
-        <v>SUGAR</v>
+        <v>MEMORIES</v>
       </c>
     </row>
     <row r="31">
@@ -837,10 +837,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C31" t="str">
-        <v>¿Qué canción de 2019 es un brindis por los seres queridos que ya no están?</v>
+        <v>¿Qué éxito de 2014 se titula «mapas» en inglés?</v>
       </c>
       <c r="D31" t="str">
-        <v>MEMORIES</v>
+        <v>MAPS</v>
       </c>
     </row>
     <row r="32">
@@ -851,10 +851,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C32" t="str">
-        <v>¿Qué éxito de 2014 se titula «mapas» en inglés?</v>
+        <v>¿Qué éxito de 2014 se titula «animales» en inglés?</v>
       </c>
       <c r="D32" t="str">
-        <v>MAPS</v>
+        <v>ANIMALS</v>
       </c>
     </row>
     <row r="33">
@@ -865,10 +865,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C33" t="str">
-        <v>¿Qué éxito de 2014 se titula «animales» en inglés?</v>
+        <v>¿Qué canción de 2010 se titula «miseria» en inglés?</v>
       </c>
       <c r="D33" t="str">
-        <v>ANIMALS</v>
+        <v>MISERY</v>
       </c>
     </row>
     <row r="34">
@@ -879,10 +879,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C34" t="str">
-        <v>¿Qué canción de 2010 se titula «miseria» en inglés?</v>
+        <v>¿Qué canción de 2012 se titula «luz del día» en inglés?</v>
       </c>
       <c r="D34" t="str">
-        <v>MISERY</v>
+        <v>DAYLIGHT</v>
       </c>
     </row>
     <row r="35">
@@ -893,10 +893,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C35" t="str">
-        <v>¿Qué canción de 2012 se titula «luz del día» en inglés?</v>
+        <v>Su vocalista fue coach durante años del programa de talentos The ___</v>
       </c>
       <c r="D35" t="str">
-        <v>DAYLIGHT</v>
+        <v>VOICE</v>
       </c>
     </row>
     <row r="36">
@@ -907,10 +907,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C36" t="str">
-        <v>Adam Levine fue coach durante años del programa de talentos The ___</v>
+        <v>En 2019 la banda encabezó el show de medio tiempo del Super ___</v>
       </c>
       <c r="D36" t="str">
-        <v>VOICE</v>
+        <v>BOWL</v>
       </c>
     </row>
     <row r="37">
@@ -921,24 +921,24 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C37" t="str">
-        <v>En 2019 Maroon 5 encabezó el show de medio tiempo del Super ___</v>
+        <v>Su disco de 2021 lleva el apodo de su mánager fallecido, Jordan Feldstein: ___</v>
       </c>
       <c r="D37" t="str">
-        <v>BOWL</v>
+        <v>JORDI</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MAROON 5</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B38" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C38" t="str">
-        <v>Su disco de 2021 lleva el apodo de su mánager fallecido, Jordan Feldstein: ___</v>
+        <v>Corazón ___</v>
       </c>
       <c r="D38" t="str">
-        <v>JORDI</v>
+        <v>PARTÍO</v>
       </c>
     </row>
     <row r="39">
@@ -949,10 +949,10 @@
         <v>CANCION</v>
       </c>
       <c r="C39" t="str">
-        <v>Corazón ___</v>
+        <v>Amiga ___</v>
       </c>
       <c r="D39" t="str">
-        <v>PARTÍO</v>
+        <v>MÍA</v>
       </c>
     </row>
     <row r="40">
@@ -963,10 +963,10 @@
         <v>CANCION</v>
       </c>
       <c r="C40" t="str">
-        <v>Amiga ___</v>
+        <v>Y si fuera ___</v>
       </c>
       <c r="D40" t="str">
-        <v>MÍA</v>
+        <v>ELLA</v>
       </c>
     </row>
     <row r="41">
@@ -977,10 +977,10 @@
         <v>CANCION</v>
       </c>
       <c r="C41" t="str">
-        <v>Y si fuera ___</v>
+        <v>Mi soledad y ___</v>
       </c>
       <c r="D41" t="str">
-        <v>ELLA</v>
+        <v>YO</v>
       </c>
     </row>
     <row r="42">
@@ -991,10 +991,10 @@
         <v>CANCION</v>
       </c>
       <c r="C42" t="str">
-        <v>Mi soledad y ___</v>
+        <v>Cuando nadie me ___</v>
       </c>
       <c r="D42" t="str">
-        <v>YO</v>
+        <v>VE</v>
       </c>
     </row>
     <row r="43">
@@ -1005,10 +1005,10 @@
         <v>CANCION</v>
       </c>
       <c r="C43" t="str">
-        <v>Cuando nadie me ___</v>
+        <v>Pisando ___</v>
       </c>
       <c r="D43" t="str">
-        <v>VE</v>
+        <v>FUERTE</v>
       </c>
     </row>
     <row r="44">
@@ -1019,10 +1019,10 @@
         <v>CANCION</v>
       </c>
       <c r="C44" t="str">
-        <v>Pisando ___</v>
+        <v>Los dos cogidos de la ___</v>
       </c>
       <c r="D44" t="str">
-        <v>FUERTE</v>
+        <v>MANO</v>
       </c>
     </row>
     <row r="45">
@@ -1033,10 +1033,10 @@
         <v>CANCION</v>
       </c>
       <c r="C45" t="str">
-        <v>Los dos cogidos de la ___</v>
+        <v>Deja que te ___</v>
       </c>
       <c r="D45" t="str">
-        <v>MANO</v>
+        <v>BESE</v>
       </c>
     </row>
     <row r="46">
@@ -1047,10 +1047,10 @@
         <v>CANCION</v>
       </c>
       <c r="C46" t="str">
-        <v>Deja que te ___</v>
+        <v>Hoy llueve, hoy ___</v>
       </c>
       <c r="D46" t="str">
-        <v>BESE</v>
+        <v>DUELE</v>
       </c>
     </row>
     <row r="47">
@@ -1061,10 +1061,10 @@
         <v>CANCION</v>
       </c>
       <c r="C47" t="str">
-        <v>Hoy llueve, hoy ___</v>
+        <v>No me ___</v>
       </c>
       <c r="D47" t="str">
-        <v>DUELE</v>
+        <v>COMPARES</v>
       </c>
     </row>
     <row r="48">
@@ -1075,10 +1075,10 @@
         <v>CANCION</v>
       </c>
       <c r="C48" t="str">
-        <v>No me ___</v>
+        <v>Mi persona ___</v>
       </c>
       <c r="D48" t="str">
-        <v>COMPARES</v>
+        <v>FAVORITA</v>
       </c>
     </row>
     <row r="49">
@@ -1089,10 +1089,10 @@
         <v>CANCION</v>
       </c>
       <c r="C49" t="str">
-        <v>Mi persona ___</v>
+        <v>Looking for ___</v>
       </c>
       <c r="D49" t="str">
-        <v>FAVORITA</v>
+        <v>PARADISE</v>
       </c>
     </row>
     <row r="50">
@@ -1103,10 +1103,10 @@
         <v>CANCION</v>
       </c>
       <c r="C50" t="str">
-        <v>Looking for ___</v>
+        <v>Siempre es de ___</v>
       </c>
       <c r="D50" t="str">
-        <v>PARADISE</v>
+        <v>NOCHE</v>
       </c>
     </row>
     <row r="51">
@@ -1117,10 +1117,10 @@
         <v>CANCION</v>
       </c>
       <c r="C51" t="str">
-        <v>Siempre es de ___</v>
+        <v>Quisiera ___</v>
       </c>
       <c r="D51" t="str">
-        <v>NOCHE</v>
+        <v>SER</v>
       </c>
     </row>
     <row r="52">
@@ -1131,10 +1131,10 @@
         <v>CANCION</v>
       </c>
       <c r="C52" t="str">
-        <v>Quisiera ___</v>
+        <v>Desde ___</v>
       </c>
       <c r="D52" t="str">
-        <v>SER</v>
+        <v>CUÁNDO</v>
       </c>
     </row>
     <row r="53">
@@ -1145,10 +1145,10 @@
         <v>CANCION</v>
       </c>
       <c r="C53" t="str">
-        <v>Desde ___</v>
+        <v>Si hay ___</v>
       </c>
       <c r="D53" t="str">
-        <v>CUÁNDO</v>
+        <v>DIOS</v>
       </c>
     </row>
     <row r="54">
@@ -1159,10 +1159,10 @@
         <v>CANCION</v>
       </c>
       <c r="C54" t="str">
-        <v>Si hay ___</v>
+        <v>Te lo agradezco, pero ___</v>
       </c>
       <c r="D54" t="str">
-        <v>DIOS</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="55">
@@ -1170,13 +1170,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B55" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C55" t="str">
-        <v>Te lo agradezco, pero ___</v>
+        <v>El alma al ___</v>
       </c>
       <c r="D55" t="str">
-        <v>NO</v>
+        <v>AIRE</v>
       </c>
     </row>
     <row r="56">
@@ -1187,10 +1187,10 @@
         <v>DISCO</v>
       </c>
       <c r="C56" t="str">
-        <v>El alma al ___</v>
+        <v>No es lo ___</v>
       </c>
       <c r="D56" t="str">
-        <v>AIRE</v>
+        <v>MISMO</v>
       </c>
     </row>
     <row r="57">
@@ -1201,10 +1201,10 @@
         <v>DISCO</v>
       </c>
       <c r="C57" t="str">
-        <v>No es lo ___</v>
+        <v>Viviendo ___</v>
       </c>
       <c r="D57" t="str">
-        <v>MISMO</v>
+        <v>DEPRISA</v>
       </c>
     </row>
     <row r="58">
@@ -1215,10 +1215,10 @@
         <v>DISCO</v>
       </c>
       <c r="C58" t="str">
-        <v>Viviendo ___</v>
+        <v>El tren de los ___</v>
       </c>
       <c r="D58" t="str">
-        <v>DEPRISA</v>
+        <v>MOMENTOS</v>
       </c>
     </row>
     <row r="59">
@@ -1229,10 +1229,10 @@
         <v>DISCO</v>
       </c>
       <c r="C59" t="str">
-        <v>El tren de los ___</v>
+        <v>La música no se ___</v>
       </c>
       <c r="D59" t="str">
-        <v>MOMENTOS</v>
+        <v>TOCA</v>
       </c>
     </row>
     <row r="60">
@@ -1243,10 +1243,10 @@
         <v>DISCO</v>
       </c>
       <c r="C60" t="str">
-        <v>La música no se ___</v>
+        <v>Paraíso ___</v>
       </c>
       <c r="D60" t="str">
-        <v>TOCA</v>
+        <v>EXPRESS</v>
       </c>
     </row>
     <row r="61">
@@ -1257,10 +1257,10 @@
         <v>DISCO</v>
       </c>
       <c r="C61" t="str">
-        <v>Paraíso ___</v>
+        <v>Si tú me ___</v>
       </c>
       <c r="D61" t="str">
-        <v>EXPRESS</v>
+        <v>MIRAS</v>
       </c>
     </row>
     <row r="62">
@@ -1268,13 +1268,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B62" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C62" t="str">
-        <v>Si tú me ___</v>
+        <v>¿Cómo se llama su disco de 1997, el de «Corazón partío»?</v>
       </c>
       <c r="D62" t="str">
-        <v>MIRAS</v>
+        <v>MÁS</v>
       </c>
     </row>
     <row r="63">
@@ -1285,10 +1285,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C63" t="str">
-        <v>¿Cómo se llama su disco de 1997, el de «Corazón partío»?</v>
+        <v>Su disco de 2015 se llama como un jarabe dulce: ___</v>
       </c>
       <c r="D63" t="str">
-        <v>MÁS</v>
+        <v>SIROPE</v>
       </c>
     </row>
     <row r="64">
@@ -1299,10 +1299,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C64" t="str">
-        <v>Su disco de 2015 se llama como un jarabe dulce: ___</v>
+        <v>Su disco de 2019 tiene nombre de hashtag: #El___</v>
       </c>
       <c r="D64" t="str">
-        <v>SIROPE</v>
+        <v>DISCO</v>
       </c>
     </row>
     <row r="65">
@@ -1313,10 +1313,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C65" t="str">
-        <v>Su disco de 2019 tiene nombre de hashtag: #El___</v>
+        <v>La canción que grabó con Shakira en 2005 se llama La ___</v>
       </c>
       <c r="D65" t="str">
-        <v>DISCO</v>
+        <v>TORTURA</v>
       </c>
     </row>
     <row r="66">
@@ -1327,10 +1327,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C66" t="str">
-        <v>Su disco de 2021 lleva su apellido artístico: ___</v>
+        <v>«Mi persona favorita» la grabó con la cantante Camila ___</v>
       </c>
       <c r="D66" t="str">
-        <v>SANZ</v>
+        <v>CABELLO</v>
       </c>
     </row>
     <row r="67">
@@ -1341,10 +1341,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C67" t="str">
-        <v>La canción que grabó con Shakira en 2005 se llama La ___</v>
+        <v>«Looking for Paradise» la grabó con la cantante Alicia ___</v>
       </c>
       <c r="D67" t="str">
-        <v>TORTURA</v>
+        <v>KEYS</v>
       </c>
     </row>
     <row r="68">
@@ -1355,10 +1355,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C68" t="str">
-        <v>«Mi persona favorita» la grabó con la cantante Camila ___</v>
+        <v>«Deja que te bese» la grabó con el cantante Marc ___</v>
       </c>
       <c r="D68" t="str">
-        <v>CABELLO</v>
+        <v>ANTHONY</v>
       </c>
     </row>
     <row r="69">
@@ -1369,10 +1369,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C69" t="str">
-        <v>«Looking for Paradise» la grabó con la cantante Alicia ___</v>
+        <v>¿En qué ciudad nació el cantante?</v>
       </c>
       <c r="D69" t="str">
-        <v>KEYS</v>
+        <v>MADRID</v>
       </c>
     </row>
     <row r="70">
@@ -1383,10 +1383,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C70" t="str">
-        <v>«Deja que te bese» la grabó con el cantante Marc ___</v>
+        <v>¿De qué país es el cantante?</v>
       </c>
       <c r="D70" t="str">
-        <v>ANTHONY</v>
+        <v>ESPAÑA</v>
       </c>
     </row>
     <row r="71">
@@ -1397,52 +1397,52 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C71" t="str">
-        <v>¿En qué ciudad nació Alejandro Sanz?</v>
+        <v>¿Qué género musical andaluz se escucha en muchas de sus canciones?</v>
       </c>
       <c r="D71" t="str">
-        <v>MADRID</v>
+        <v>FLAMENCO</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B72" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C72" t="str">
-        <v>¿De qué país es Alejandro Sanz?</v>
+        <v>¿Y todo para ___?</v>
       </c>
       <c r="D72" t="str">
-        <v>ESPAÑA</v>
+        <v>QUÉ</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B73" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C73" t="str">
-        <v>¿Qué género musical andaluz se escucha en muchas de sus canciones?</v>
+        <v>Enséñame a ___</v>
       </c>
       <c r="D73" t="str">
-        <v>FLAMENCO</v>
+        <v>OLVIDAR</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B74" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C74" t="str">
-        <v>Su nombre real es Alejandro Sánchez ___</v>
+        <v>Alguien te va a hacer ___</v>
       </c>
       <c r="D74" t="str">
-        <v>PIZARRO</v>
+        <v>LLORAR</v>
       </c>
     </row>
     <row r="75">
@@ -1453,10 +1453,10 @@
         <v>CANCION</v>
       </c>
       <c r="C75" t="str">
-        <v>¿Y todo para ___?</v>
+        <v>¿Dónde ___?</v>
       </c>
       <c r="D75" t="str">
-        <v>QUÉ</v>
+        <v>ESTÁS</v>
       </c>
     </row>
     <row r="76">
@@ -1467,10 +1467,10 @@
         <v>CANCION</v>
       </c>
       <c r="C76" t="str">
-        <v>Enséñame a ___</v>
+        <v>Fuerte no ___</v>
       </c>
       <c r="D76" t="str">
-        <v>OLVIDAR</v>
+        <v>SOY</v>
       </c>
     </row>
     <row r="77">
@@ -1478,13 +1478,13 @@
         <v>INTOCABLE</v>
       </c>
       <c r="B77" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C77" t="str">
-        <v>Alguien te va a hacer ___</v>
+        <v>Nuestro destino estaba ___</v>
       </c>
       <c r="D77" t="str">
-        <v>LLORAR</v>
+        <v>ESCRITO</v>
       </c>
     </row>
     <row r="78">
@@ -1492,13 +1492,13 @@
         <v>INTOCABLE</v>
       </c>
       <c r="B78" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C78" t="str">
-        <v>¿Dónde ___?</v>
+        <v>¿Qué instrumento toca el vocalista del grupo mientras canta?</v>
       </c>
       <c r="D78" t="str">
-        <v>ESTÁS</v>
+        <v>ACORDEÓN</v>
       </c>
     </row>
     <row r="79">
@@ -1506,13 +1506,13 @@
         <v>INTOCABLE</v>
       </c>
       <c r="B79" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C79" t="str">
-        <v>Fuerte no ___</v>
+        <v>¿De qué estado de Estados Unidos es el grupo?</v>
       </c>
       <c r="D79" t="str">
-        <v>SOY</v>
+        <v>TEXAS</v>
       </c>
     </row>
     <row r="80">
@@ -1520,13 +1520,13 @@
         <v>INTOCABLE</v>
       </c>
       <c r="B80" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C80" t="str">
-        <v>Nuestro destino estaba ___</v>
+        <v>¿En qué pueblo de Texas nació el grupo?</v>
       </c>
       <c r="D80" t="str">
-        <v>ESCRITO</v>
+        <v>ZAPATA</v>
       </c>
     </row>
     <row r="81">
@@ -1537,10 +1537,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C81" t="str">
-        <v>¿Cómo se apellida Ricky, el vocalista y acordeonista de Intocable?</v>
+        <v>La guitarra de doce cuerdas típica del norteño se llama bajo ___</v>
       </c>
       <c r="D81" t="str">
-        <v>MUÑOZ</v>
+        <v>SEXTO</v>
       </c>
     </row>
     <row r="82">
@@ -1551,66 +1551,66 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C82" t="str">
-        <v>¿Qué instrumento toca Ricky Muñoz mientras canta?</v>
+        <v>¿Cómo se llama la música de los mexicanos de Texas que toca el grupo?</v>
       </c>
       <c r="D82" t="str">
-        <v>ACORDEÓN</v>
+        <v>TEJANO</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>INTOCABLE</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B83" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C83" t="str">
-        <v>¿De qué estado de Estados Unidos es Intocable?</v>
+        <v>Al acordeonista Ramón Ayala le dicen el Rey del ___</v>
       </c>
       <c r="D83" t="str">
-        <v>TEXAS</v>
+        <v>ACORDEÓN</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>INTOCABLE</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B84" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C84" t="str">
-        <v>¿En qué pueblo de Texas nació Intocable?</v>
+        <v>«Tragos amargos» es un clásico de Ramón ___</v>
       </c>
       <c r="D84" t="str">
-        <v>ZAPATA</v>
+        <v>AYALA</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>INTOCABLE</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B85" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C85" t="str">
-        <v>La guitarra de doce cuerdas típica del norteño se llama bajo ___</v>
+        <v>«La puerta negra» es de Los Tigres del ___</v>
       </c>
       <c r="D85" t="str">
-        <v>SEXTO</v>
+        <v>NORTE</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>INTOCABLE</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B86" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C86" t="str">
-        <v>¿Cómo se llama la música de los mexicanos de Texas que toca Intocable?</v>
+        <v>«Contrabando y traición» es de Los Tigres del ___</v>
       </c>
       <c r="D86" t="str">
-        <v>TEJANO</v>
+        <v>NORTE</v>
       </c>
     </row>
     <row r="87">
@@ -1621,10 +1621,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C87" t="str">
-        <v>Al acordeonista Ramón Ayala le dicen el Rey del ___</v>
+        <v>«Me caí de la nube» es un clásico de Cornelio ___</v>
       </c>
       <c r="D87" t="str">
-        <v>ACORDEÓN</v>
+        <v>REYNA</v>
       </c>
     </row>
     <row r="88">
@@ -1635,10 +1635,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C88" t="str">
-        <v>«Tragos amargos» es un clásico de Ramón ___</v>
+        <v>«Laurita Garza» es de Los Invasores de Nuevo ___</v>
       </c>
       <c r="D88" t="str">
-        <v>AYALA</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="89">
@@ -1649,7 +1649,7 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C89" t="str">
-        <v>«La puerta negra» es de Los Tigres del ___</v>
+        <v>Ramón Ayala y Cornelio Reyna formaron Los Relámpagos del ___</v>
       </c>
       <c r="D89" t="str">
         <v>NORTE</v>
@@ -1663,10 +1663,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C90" t="str">
-        <v>«Contrabando y traición» es de Los Tigres del ___</v>
+        <v>¿Cómo le dicen a Selena? La reina del Tex-___</v>
       </c>
       <c r="D90" t="str">
-        <v>NORTE</v>
+        <v>MEX</v>
       </c>
     </row>
     <row r="91">
@@ -1677,10 +1677,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C91" t="str">
-        <v>«Me caí de la nube» es un clásico de Cornelio ___</v>
+        <v>¿Qué baile europeo, de ritmo rápido, está en las raíces del norteño?</v>
       </c>
       <c r="D91" t="str">
-        <v>REYNA</v>
+        <v>POLKA</v>
       </c>
     </row>
     <row r="92">
@@ -1691,66 +1691,66 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C92" t="str">
-        <v>«Laurita Garza» es de Los Invasores de Nuevo ___</v>
+        <v>¿De qué ciudad es el grupo norteño Pesado?</v>
       </c>
       <c r="D92" t="str">
-        <v>LEÓN</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>NORTEÑO</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B93" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C93" t="str">
-        <v>Ramón Ayala y Cornelio Reyna formaron Los Relámpagos del ___</v>
+        <v>Da Ya Think I'm ___?</v>
       </c>
       <c r="D93" t="str">
-        <v>NORTE</v>
+        <v>SEXY</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>NORTEÑO</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B94" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C94" t="str">
-        <v>¿Cómo le dicen a Selena? La reina del Tex-___</v>
+        <v>Maggie ___</v>
       </c>
       <c r="D94" t="str">
-        <v>MEX</v>
+        <v>MAY</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>NORTEÑO</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B95" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C95" t="str">
-        <v>¿Qué baile europeo, de ritmo rápido, está en las raíces del norteño?</v>
+        <v>Young ___</v>
       </c>
       <c r="D95" t="str">
-        <v>POLKA</v>
+        <v>TURKS</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>NORTEÑO</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B96" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C96" t="str">
-        <v>¿De qué ciudad es el grupo norteño Pesado?</v>
+        <v>Have I Told You ___</v>
       </c>
       <c r="D96" t="str">
-        <v>MONTERREY</v>
+        <v>LATELY</v>
       </c>
     </row>
     <row r="97">
@@ -1761,10 +1761,10 @@
         <v>CANCION</v>
       </c>
       <c r="C97" t="str">
-        <v>Da Ya Think I'm ___?</v>
+        <v>Forever ___</v>
       </c>
       <c r="D97" t="str">
-        <v>SEXY</v>
+        <v>YOUNG</v>
       </c>
     </row>
     <row r="98">
@@ -1775,10 +1775,10 @@
         <v>CANCION</v>
       </c>
       <c r="C98" t="str">
-        <v>Maggie ___</v>
+        <v>Some Guys Have All the ___</v>
       </c>
       <c r="D98" t="str">
-        <v>MAY</v>
+        <v>LUCK</v>
       </c>
     </row>
     <row r="99">
@@ -1789,10 +1789,10 @@
         <v>CANCION</v>
       </c>
       <c r="C99" t="str">
-        <v>Young ___</v>
+        <v>Hot ___</v>
       </c>
       <c r="D99" t="str">
-        <v>TURKS</v>
+        <v>LEGS</v>
       </c>
     </row>
     <row r="100">
@@ -1803,10 +1803,10 @@
         <v>CANCION</v>
       </c>
       <c r="C100" t="str">
-        <v>Have I Told You ___</v>
+        <v>Tonight's the ___</v>
       </c>
       <c r="D100" t="str">
-        <v>LATELY</v>
+        <v>NIGHT</v>
       </c>
     </row>
     <row r="101">
@@ -1817,10 +1817,10 @@
         <v>CANCION</v>
       </c>
       <c r="C101" t="str">
-        <v>Forever ___</v>
+        <v>Baby ___</v>
       </c>
       <c r="D101" t="str">
-        <v>YOUNG</v>
+        <v>JANE</v>
       </c>
     </row>
     <row r="102">
@@ -1831,10 +1831,10 @@
         <v>CANCION</v>
       </c>
       <c r="C102" t="str">
-        <v>Some Guys Have All the ___</v>
+        <v>Downtown ___</v>
       </c>
       <c r="D102" t="str">
-        <v>LUCK</v>
+        <v>TRAIN</v>
       </c>
     </row>
     <row r="103">
@@ -1845,10 +1845,10 @@
         <v>CANCION</v>
       </c>
       <c r="C103" t="str">
-        <v>Hot ___</v>
+        <v>Rhythm of My ___</v>
       </c>
       <c r="D103" t="str">
-        <v>LEGS</v>
+        <v>HEART</v>
       </c>
     </row>
     <row r="104">
@@ -1859,10 +1859,10 @@
         <v>CANCION</v>
       </c>
       <c r="C104" t="str">
-        <v>Tonight's the ___</v>
+        <v>The First ___ Is the Deepest</v>
       </c>
       <c r="D104" t="str">
-        <v>NIGHT</v>
+        <v>CUT</v>
       </c>
     </row>
     <row r="105">
@@ -1873,10 +1873,10 @@
         <v>CANCION</v>
       </c>
       <c r="C105" t="str">
-        <v>Baby ___</v>
+        <v>You Wear It ___</v>
       </c>
       <c r="D105" t="str">
-        <v>JANE</v>
+        <v>WELL</v>
       </c>
     </row>
     <row r="106">
@@ -1887,10 +1887,10 @@
         <v>CANCION</v>
       </c>
       <c r="C106" t="str">
-        <v>Downtown ___</v>
+        <v>I Don't Want to Talk About ___</v>
       </c>
       <c r="D106" t="str">
-        <v>TRAIN</v>
+        <v>IT</v>
       </c>
     </row>
     <row r="107">
@@ -1901,10 +1901,10 @@
         <v>CANCION</v>
       </c>
       <c r="C107" t="str">
-        <v>Rhythm of My ___</v>
+        <v>Reason to ___</v>
       </c>
       <c r="D107" t="str">
-        <v>HEART</v>
+        <v>BELIEVE</v>
       </c>
     </row>
     <row r="108">
@@ -1915,10 +1915,10 @@
         <v>CANCION</v>
       </c>
       <c r="C108" t="str">
-        <v>The First ___ Is the Deepest</v>
+        <v>All for ___</v>
       </c>
       <c r="D108" t="str">
-        <v>CUT</v>
+        <v>LOVE</v>
       </c>
     </row>
     <row r="109">
@@ -1926,13 +1926,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B109" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C109" t="str">
-        <v>You Wear It ___</v>
+        <v>Every Picture Tells a ___</v>
       </c>
       <c r="D109" t="str">
-        <v>WELL</v>
+        <v>STORY</v>
       </c>
     </row>
     <row r="110">
@@ -1940,13 +1940,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B110" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C110" t="str">
-        <v>I Don't Want to Talk About ___</v>
+        <v>Atlantic ___</v>
       </c>
       <c r="D110" t="str">
-        <v>IT</v>
+        <v>CROSSING</v>
       </c>
     </row>
     <row r="111">
@@ -1954,13 +1954,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B111" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C111" t="str">
-        <v>Reason to ___</v>
+        <v>Blondes Have More ___</v>
       </c>
       <c r="D111" t="str">
-        <v>BELIEVE</v>
+        <v>FUN</v>
       </c>
     </row>
     <row r="112">
@@ -1968,13 +1968,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B112" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C112" t="str">
-        <v>All for ___</v>
+        <v>A Night on the ___</v>
       </c>
       <c r="D112" t="str">
-        <v>LOVE</v>
+        <v>TOWN</v>
       </c>
     </row>
     <row r="113">
@@ -1985,10 +1985,10 @@
         <v>DISCO</v>
       </c>
       <c r="C113" t="str">
-        <v>Every Picture Tells a ___</v>
+        <v>Gasoline ___</v>
       </c>
       <c r="D113" t="str">
-        <v>STORY</v>
+        <v>ALLEY</v>
       </c>
     </row>
     <row r="114">
@@ -1996,13 +1996,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B114" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C114" t="str">
-        <v>Atlantic ___</v>
+        <v>¿Qué canción de 1975 habla de navegar por el mar?</v>
       </c>
       <c r="D114" t="str">
-        <v>CROSSING</v>
+        <v>SAILING</v>
       </c>
     </row>
     <row r="115">
@@ -2010,13 +2010,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B115" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C115" t="str">
-        <v>Blondes Have More ___</v>
+        <v>Antes de ser solista, cantó en la banda The ___</v>
       </c>
       <c r="D115" t="str">
-        <v>FUN</v>
+        <v>FACES</v>
       </c>
     </row>
     <row r="116">
@@ -2024,13 +2024,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B116" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C116" t="str">
-        <v>A Night on the ___</v>
+        <v>Su primer grupo famoso lo formó con el guitarrista Jeff ___</v>
       </c>
       <c r="D116" t="str">
-        <v>TOWN</v>
+        <v>BECK</v>
       </c>
     </row>
     <row r="117">
@@ -2038,13 +2038,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B117" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C117" t="str">
-        <v>Gasoline ___</v>
+        <v>En los años 60 lo apodaban «Rod the ___»</v>
       </c>
       <c r="D117" t="str">
-        <v>ALLEY</v>
+        <v>MOD</v>
       </c>
     </row>
     <row r="118">
@@ -2055,10 +2055,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C118" t="str">
-        <v>¿Qué canción de 1975 habla de navegar por el mar?</v>
+        <v>¿En qué ciudad nació el cantante?</v>
       </c>
       <c r="D118" t="str">
-        <v>SAILING</v>
+        <v>LONDRES</v>
       </c>
     </row>
     <row r="119">
@@ -2069,10 +2069,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C119" t="str">
-        <v>Antes de ser solista, cantó en la banda The ___</v>
+        <v>¿De qué país es su familia paterna, al que siempre dice pertenecer?</v>
       </c>
       <c r="D119" t="str">
-        <v>FACES</v>
+        <v>ESCOCIA</v>
       </c>
     </row>
     <row r="120">
@@ -2083,10 +2083,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C120" t="str">
-        <v>Su primer grupo famoso lo formó con el guitarrista Jeff ___</v>
+        <v>¿De qué equipo de futbol escocés es fanático el cantante?</v>
       </c>
       <c r="D120" t="str">
-        <v>BECK</v>
+        <v>CELTIC</v>
       </c>
     </row>
     <row r="121">
@@ -2097,10 +2097,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C121" t="str">
-        <v>En los años 60 lo apodaban «Rod the ___»</v>
+        <v>Su serie de discos de clásicos se llama The Great American ___</v>
       </c>
       <c r="D121" t="str">
-        <v>MOD</v>
+        <v>SONGBOOK</v>
       </c>
     </row>
     <row r="122">
@@ -2111,10 +2111,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C122" t="str">
-        <v>¿En qué ciudad nació Rod Stewart?</v>
+        <v>Desde 2016 es caballero británico, así que antes de su nombre lleva el título de ___</v>
       </c>
       <c r="D122" t="str">
-        <v>LONDRES</v>
+        <v>SIR</v>
       </c>
     </row>
     <row r="123">
@@ -2125,10 +2125,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C123" t="str">
-        <v>¿De qué país es su familia paterna, al que siempre dice pertenecer?</v>
+        <v>«All for Love» la grabó con Bryan Adams y ___</v>
       </c>
       <c r="D123" t="str">
-        <v>ESCOCIA</v>
+        <v>STING</v>
       </c>
     </row>
     <row r="124">
@@ -2139,10 +2139,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C124" t="str">
-        <v>¿De qué equipo de futbol escocés es fanático Rod Stewart?</v>
+        <v>¿En qué playa de Río de Janeiro dio un concierto histórico en 1994?</v>
       </c>
       <c r="D124" t="str">
-        <v>CELTIC</v>
+        <v>COPACABANA</v>
       </c>
     </row>
     <row r="125">
@@ -2153,66 +2153,66 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C125" t="str">
-        <v>Su serie de discos de clásicos se llama The Great American ___</v>
+        <v>Su gran pasatiempo es armar maquetas gigantes de ___</v>
       </c>
       <c r="D125" t="str">
-        <v>SONGBOOK</v>
+        <v>TRENES</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>ROD STEWART</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B126" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C126" t="str">
-        <v>Desde que lo nombraron caballero en 2016 le dicen ___ Rod Stewart</v>
+        <v>Ella quiere ___</v>
       </c>
       <c r="D126" t="str">
-        <v>SIR</v>
+        <v>BEBER</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>ROD STEWART</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B127" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C127" t="str">
-        <v>«All for Love» la grabó con Bryan Adams y ___</v>
+        <v>Hasta que Dios ___</v>
       </c>
       <c r="D127" t="str">
-        <v>STING</v>
+        <v>DIGA</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>ROD STEWART</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B128" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C128" t="str">
-        <v>¿En qué playa de Río de Janeiro dio un concierto histórico en 1994?</v>
+        <v>Mejor que ___</v>
       </c>
       <c r="D128" t="str">
-        <v>COPACABANA</v>
+        <v>YO</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>ROD STEWART</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B129" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C129" t="str">
-        <v>Su gran pasatiempo es armar maquetas gigantes de ___</v>
+        <v>Las leyendas nunca ___</v>
       </c>
       <c r="D129" t="str">
-        <v>TRENES</v>
+        <v>MUEREN</v>
       </c>
     </row>
     <row r="130">
@@ -2220,13 +2220,13 @@
         <v>ANUEL AA</v>
       </c>
       <c r="B130" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C130" t="str">
-        <v>Ella quiere ___</v>
+        <v>Su disco con Ozuna se llama Los ___</v>
       </c>
       <c r="D130" t="str">
-        <v>BEBER</v>
+        <v>DIOSES</v>
       </c>
     </row>
     <row r="131">
@@ -2234,13 +2234,13 @@
         <v>ANUEL AA</v>
       </c>
       <c r="B131" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C131" t="str">
-        <v>Hasta que Dios ___</v>
+        <v>El cantante nació en Carolina, Puerto ___</v>
       </c>
       <c r="D131" t="str">
-        <v>DIGA</v>
+        <v>RICO</v>
       </c>
     </row>
     <row r="132">
@@ -2248,13 +2248,13 @@
         <v>ANUEL AA</v>
       </c>
       <c r="B132" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C132" t="str">
-        <v>Mejor que ___</v>
+        <v>¿Con qué cantante puertorriqueño grabó el disco «Los Dioses»?</v>
       </c>
       <c r="D132" t="str">
-        <v>YO</v>
+        <v>OZUNA</v>
       </c>
     </row>
     <row r="133">
@@ -2262,13 +2262,13 @@
         <v>ANUEL AA</v>
       </c>
       <c r="B133" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C133" t="str">
-        <v>Las leyendas nunca ___</v>
+        <v>¿Qué canción de 2019 grabó con Karol G?</v>
       </c>
       <c r="D133" t="str">
-        <v>MUEREN</v>
+        <v>SECRETO</v>
       </c>
     </row>
     <row r="134">
@@ -2279,10 +2279,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C134" t="str">
-        <v>Su disco con Ozuna se llama Los ___</v>
+        <v>¿Qué canción de 2019 grabó junto a Daddy Yankee, Karol G, Ozuna y J Balvin?</v>
       </c>
       <c r="D134" t="str">
-        <v>DIOSES</v>
+        <v>CHINA</v>
       </c>
     </row>
     <row r="135">
@@ -2293,10 +2293,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C135" t="str">
-        <v>¿Cómo se llama su disco de 2020, que lleva su primer nombre?</v>
+        <v>¿Qué canción grabó con Tekashi 6ix9ine en 2018?</v>
       </c>
       <c r="D135" t="str">
-        <v>EMMANUEL</v>
+        <v>BEBÉ</v>
       </c>
     </row>
     <row r="136">
@@ -2307,10 +2307,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C136" t="str">
-        <v>Su nombre real es Emmanuel ___ Santiago</v>
+        <v>¿Cómo se llama su primer gran éxito, de 2016?</v>
       </c>
       <c r="D136" t="str">
-        <v>GAZMEY</v>
+        <v>SOLA</v>
       </c>
     </row>
     <row r="137">
@@ -2321,10 +2321,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C137" t="str">
-        <v>Anuel AA nació en Carolina, Puerto ___</v>
+        <v>El remix de «Sola» lo grabó con Daddy Yankee, Wisin, Farruko y Zion &amp; ___</v>
       </c>
       <c r="D137" t="str">
-        <v>RICO</v>
+        <v>LENNOX</v>
       </c>
     </row>
     <row r="138">
@@ -2335,10 +2335,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C138" t="str">
-        <v>¿Con qué cantante puertorriqueño grabó el disco «Los Dioses»?</v>
+        <v>«Adicto» la grabó con Ozuna y el productor ___</v>
       </c>
       <c r="D138" t="str">
-        <v>OZUNA</v>
+        <v>TAINY</v>
       </c>
     </row>
     <row r="139">
@@ -2349,10 +2349,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C139" t="str">
-        <v>¿Qué canción de 2019 grabó con Karol G?</v>
+        <v>«Hasta que Dios diga» la grabó con Bad ___</v>
       </c>
       <c r="D139" t="str">
-        <v>SECRETO</v>
+        <v>BUNNY</v>
       </c>
     </row>
     <row r="140">
@@ -2363,94 +2363,94 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C140" t="str">
-        <v>¿Qué canción de 2019 junta a Anuel con Daddy Yankee, Karol G, Ozuna y J Balvin?</v>
+        <v>Además del reguetón, su género es el ___ latino</v>
       </c>
       <c r="D140" t="str">
-        <v>CHINA</v>
+        <v>TRAP</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B141" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C141" t="str">
-        <v>¿Qué canción grabó con Tekashi 6ix9ine en 2018?</v>
+        <v>¿Cómo se llama el estadio de Tigres? Estadio ___</v>
       </c>
       <c r="D141" t="str">
-        <v>BEBÉ</v>
+        <v>UNIVERSITARIO</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B142" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C142" t="str">
-        <v>¿Cómo se llama su primer gran éxito, de 2016?</v>
+        <v>¿Cómo le dicen al Estadio Universitario por lo caliente de su ambiente?</v>
       </c>
       <c r="D142" t="str">
-        <v>SOLA</v>
+        <v>VOLCÁN</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B143" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C143" t="str">
-        <v>El remix de «Sola» lo grabó con Daddy Yankee, Wisin, Farruko y Zion &amp; ___</v>
+        <v>El Volcán está en el municipio de San Nicolás de los ___</v>
       </c>
       <c r="D143" t="str">
-        <v>LENNOX</v>
+        <v>GARZA</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B144" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C144" t="str">
-        <v>«Adicto» la grabó con Ozuna y el productor ___</v>
+        <v>Tigres es el equipo de la Universidad Autónoma de Nuevo ___</v>
       </c>
       <c r="D144" t="str">
-        <v>TAINY</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B145" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C145" t="str">
-        <v>«Hasta que Dios diga» la grabó con Bad ___</v>
+        <v>¿En qué año se fundó Tigres?</v>
       </c>
       <c r="D145" t="str">
-        <v>BUNNY</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>ANUEL AA</v>
+        <v>TIGRES</v>
       </c>
       <c r="B146" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C146" t="str">
-        <v>Además del reguetón, su género es el ___ latino</v>
+        <v>Los colores de Tigres son el azul y el ___</v>
       </c>
       <c r="D146" t="str">
-        <v>TRAP</v>
+        <v>AMARILLO</v>
       </c>
     </row>
     <row r="147">
@@ -2461,10 +2461,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C147" t="str">
-        <v>¿Cómo se llama el estadio de Tigres? Estadio ___</v>
+        <v>Por su uniforme amarillo y azul, a Tigres también le dicen los ___</v>
       </c>
       <c r="D147" t="str">
-        <v>UNIVERSITARIO</v>
+        <v>AURIAZULES</v>
       </c>
     </row>
     <row r="148">
@@ -2475,10 +2475,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C148" t="str">
-        <v>¿Cómo le dicen al Estadio Universitario por lo caliente de su ambiente?</v>
+        <v>¿Qué animal es el emblema de la UANL?</v>
       </c>
       <c r="D148" t="str">
-        <v>VOLCÁN</v>
+        <v>TIGRE</v>
       </c>
     </row>
     <row r="149">
@@ -2489,10 +2489,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C149" t="str">
-        <v>El Volcán está en el municipio de San Nicolás de los ___</v>
+        <v>¿Cómo se apellida André-Pierre, el máximo goleador en la historia de Tigres?</v>
       </c>
       <c r="D149" t="str">
-        <v>GARZA</v>
+        <v>GIGNAC</v>
       </c>
     </row>
     <row r="150">
@@ -2503,10 +2503,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C150" t="str">
-        <v>Tigres es el equipo de la Universidad Autónoma de Nuevo ___</v>
+        <v>¿De qué país es André-Pierre Gignac?</v>
       </c>
       <c r="D150" t="str">
-        <v>LEÓN</v>
+        <v>FRANCIA</v>
       </c>
     </row>
     <row r="151">
@@ -2517,10 +2517,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C151" t="str">
-        <v>¿En qué año se fundó Tigres?</v>
+        <v>Con el técnico Ricardo «Tuca» ___, Tigres ganó cinco títulos de liga</v>
       </c>
       <c r="D151" t="str">
-        <v>1960</v>
+        <v>FERRETTI</v>
       </c>
     </row>
     <row r="152">
@@ -2531,10 +2531,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C152" t="str">
-        <v>Los colores de Tigres son el azul y el ___</v>
+        <v>¿De qué país es el técnico Ricardo «Tuca» Ferretti?</v>
       </c>
       <c r="D152" t="str">
-        <v>AMARILLO</v>
+        <v>BRASIL</v>
       </c>
     </row>
     <row r="153">
@@ -2545,10 +2545,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C153" t="str">
-        <v>Por su uniforme amarillo y azul, a Tigres también le dicen los ___</v>
+        <v>Al portero argentino Nahuel Guzmán le apodan «El ___»</v>
       </c>
       <c r="D153" t="str">
-        <v>AURIAZULES</v>
+        <v>PATÓN</v>
       </c>
     </row>
     <row r="154">
@@ -2559,10 +2559,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C154" t="str">
-        <v>¿Qué animal es el emblema de la UANL?</v>
+        <v>El mediocampista argentino que fue capitán de Tigres: Guido ___</v>
       </c>
       <c r="D154" t="str">
-        <v>TIGRE</v>
+        <v>PIZARRO</v>
       </c>
     </row>
     <row r="155">
@@ -2573,10 +2573,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C155" t="str">
-        <v>¿Cómo se apellida André-Pierre, el máximo goleador en la historia de Tigres?</v>
+        <v>En 2020 Tigres ganó la Concacaf ___ League</v>
       </c>
       <c r="D155" t="str">
-        <v>GIGNAC</v>
+        <v>CHAMPIONS</v>
       </c>
     </row>
     <row r="156">
@@ -2587,10 +2587,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C156" t="str">
-        <v>¿De qué país es André-Pierre Gignac?</v>
+        <v>En la final del Mundial de Clubes 2020, Tigres enfrentó al Bayern ___</v>
       </c>
       <c r="D156" t="str">
-        <v>FRANCIA</v>
+        <v>MÚNICH</v>
       </c>
     </row>
     <row r="157">
@@ -2601,10 +2601,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C157" t="str">
-        <v>Con el técnico Ricardo «Tuca» ___, Tigres ganó cinco títulos de liga</v>
+        <v>A la afición de Tigres se le conoce como «La afición ___»</v>
       </c>
       <c r="D157" t="str">
-        <v>FERRETTI</v>
+        <v>INCOMPARABLE</v>
       </c>
     </row>
     <row r="158">
@@ -2615,10 +2615,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C158" t="str">
-        <v>¿De qué país es el técnico Ricardo «Tuca» Ferretti?</v>
+        <v>La barra de Tigres se llama Libres y ___</v>
       </c>
       <c r="D158" t="str">
-        <v>BRASIL</v>
+        <v>LOKOS</v>
       </c>
     </row>
     <row r="159">
@@ -2629,10 +2629,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C159" t="str">
-        <v>Al portero argentino Nahuel Guzmán le apodan «El ___»</v>
+        <v>El partido entre Tigres y Rayados se llama el Clásico ___</v>
       </c>
       <c r="D159" t="str">
-        <v>PATÓN</v>
+        <v>REGIO</v>
       </c>
     </row>
     <row r="160">
@@ -2643,94 +2643,94 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C160" t="str">
-        <v>El mediocampista argentino que fue capitán de Tigres: Guido ___</v>
+        <v>¿Cómo se llama el equipo de mujeres de la UANL? Tigres ___</v>
       </c>
       <c r="D160" t="str">
-        <v>PIZARRO</v>
+        <v>FEMENIL</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B161" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C161" t="str">
-        <v>En 2020 Tigres ganó la Concacaf ___ League</v>
+        <v>¿Cómo se llama el estadio de Rayados? Estadio ___</v>
       </c>
       <c r="D161" t="str">
-        <v>CHAMPIONS</v>
+        <v>BBVA</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B162" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C162" t="str">
-        <v>En la final del Mundial de Clubes 2020, Tigres enfrentó al Bayern ___</v>
+        <v>Al Estadio BBVA le dicen el Gigante de ___</v>
       </c>
       <c r="D162" t="str">
-        <v>MÚNICH</v>
+        <v>ACERO</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B163" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C163" t="str">
-        <v>A la afición de Tigres se le conoce como «La afición ___»</v>
+        <v>¿En qué año se inauguró el Estadio BBVA?</v>
       </c>
       <c r="D163" t="str">
-        <v>INCOMPARABLE</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B164" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C164" t="str">
-        <v>La barra de Tigres se llama Libres y ___</v>
+        <v>¿En qué municipio está el Estadio BBVA?</v>
       </c>
       <c r="D164" t="str">
-        <v>LOKOS</v>
+        <v>GUADALUPE</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B165" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C165" t="str">
-        <v>El partido entre Tigres y Rayados se llama el Clásico ___</v>
+        <v>El Estadio BBVA está junto al parque ecológico La ___</v>
       </c>
       <c r="D165" t="str">
-        <v>REGIO</v>
+        <v>PASTORA</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>TIGRES</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B166" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C166" t="str">
-        <v>¿Cómo se llama el equipo de mujeres de la UANL? Tigres ___</v>
+        <v>Desde las gradas del BBVA se ve el Cerro de la ___</v>
       </c>
       <c r="D166" t="str">
-        <v>FEMENIL</v>
+        <v>SILLA</v>
       </c>
     </row>
     <row r="167">
@@ -2741,10 +2741,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C167" t="str">
-        <v>¿Cómo se llama el estadio de Rayados? Estadio ___</v>
+        <v>Antes del BBVA, Rayados jugaba de local en el Estadio ___</v>
       </c>
       <c r="D167" t="str">
-        <v>BBVA</v>
+        <v>TECNOLÓGICO</v>
       </c>
     </row>
     <row r="168">
@@ -2755,10 +2755,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C168" t="str">
-        <v>Al Estadio BBVA le dicen el Gigante de ___</v>
+        <v>El nombre oficial de Rayados es Club de Futbol ___</v>
       </c>
       <c r="D168" t="str">
-        <v>ACERO</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="169">
@@ -2769,10 +2769,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C169" t="str">
-        <v>¿En qué año se inauguró el Estadio BBVA?</v>
+        <v>¿En qué año se fundó Rayados?</v>
       </c>
       <c r="D169" t="str">
-        <v>2015</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="170">
@@ -2783,10 +2783,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C170" t="str">
-        <v>¿En qué municipio está el Estadio BBVA?</v>
+        <v>El uniforme de Rayados tiene rayas verticales azules y ___</v>
       </c>
       <c r="D170" t="str">
-        <v>GUADALUPE</v>
+        <v>BLANCAS</v>
       </c>
     </row>
     <row r="171">
@@ -2797,10 +2797,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C171" t="str">
-        <v>El Estadio BBVA está junto al parque ecológico La ___</v>
+        <v>Además de Rayados, al equipo también le dicen La ___</v>
       </c>
       <c r="D171" t="str">
-        <v>PASTORA</v>
+        <v>PANDILLA</v>
       </c>
     </row>
     <row r="172">
@@ -2811,10 +2811,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C172" t="str">
-        <v>Desde las gradas del BBVA se ve el Cerro de la ___</v>
+        <v>¿En qué año ganó Rayados su primer título de liga?</v>
       </c>
       <c r="D172" t="str">
-        <v>SILLA</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="173">
@@ -2825,10 +2825,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C173" t="str">
-        <v>Antes del BBVA, Rayados jugaba de local en el Estadio ___</v>
+        <v>Entre 2011 y 2013, ¿cuántas Concachampions seguidas ganó Rayados?</v>
       </c>
       <c r="D173" t="str">
-        <v>TECNOLÓGICO</v>
+        <v>TRES</v>
       </c>
     </row>
     <row r="174">
@@ -2839,10 +2839,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C174" t="str">
-        <v>El nombre oficial de Rayados es Club de Futbol ___</v>
+        <v>Al técnico Víctor Manuel Vucetich le dicen el Rey ___</v>
       </c>
       <c r="D174" t="str">
-        <v>MONTERREY</v>
+        <v>MIDAS</v>
       </c>
     </row>
     <row r="175">
@@ -2853,10 +2853,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C175" t="str">
-        <v>¿En qué año se fundó Rayados?</v>
+        <v>Al delantero chileno Humberto Suazo le decían «___»</v>
       </c>
       <c r="D175" t="str">
-        <v>1945</v>
+        <v>CHUPETE</v>
       </c>
     </row>
     <row r="176">
@@ -2867,10 +2867,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C176" t="str">
-        <v>El uniforme de Rayados tiene rayas verticales azules y ___</v>
+        <v>El máximo goleador en la historia de Rayados es Rogelio Funes ___</v>
       </c>
       <c r="D176" t="str">
-        <v>BLANCAS</v>
+        <v>MORI</v>
       </c>
     </row>
     <row r="177">
@@ -2881,10 +2881,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C177" t="str">
-        <v>Además de Rayados, al equipo también le dicen La ___</v>
+        <v>Al ídolo regiomontano Jesús Arellano le decían «El ___»</v>
       </c>
       <c r="D177" t="str">
-        <v>PANDILLA</v>
+        <v>CABRITO</v>
       </c>
     </row>
     <row r="178">
@@ -2895,10 +2895,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C178" t="str">
-        <v>¿En qué año ganó Rayados su primer título de liga?</v>
+        <v>En 2025 llegó a Rayados el famoso defensa español Sergio ___</v>
       </c>
       <c r="D178" t="str">
-        <v>1986</v>
+        <v>RAMOS</v>
       </c>
     </row>
     <row r="179">
@@ -2909,10 +2909,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C179" t="str">
-        <v>Entre 2011 y 2013, ¿cuántas Concachampions seguidas ganó Rayados?</v>
+        <v>Rayados quedó en tercer lugar del Mundial de ___ en 2012 y en 2019</v>
       </c>
       <c r="D179" t="str">
-        <v>TRES</v>
+        <v>CLUBES</v>
       </c>
     </row>
     <row r="180">
@@ -2923,10 +2923,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C180" t="str">
-        <v>Al técnico Víctor Manuel Vucetich le dicen el Rey ___</v>
+        <v>A la barra de Rayados se le conoce como La ___</v>
       </c>
       <c r="D180" t="str">
-        <v>MIDAS</v>
+        <v>ADICCIÓN</v>
       </c>
     </row>
     <row r="181">
@@ -2937,10 +2937,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C181" t="str">
-        <v>Al delantero chileno Humberto Suazo le decían «___»</v>
+        <v>El partido entre Rayados y Tigres se llama el Clásico ___</v>
       </c>
       <c r="D181" t="str">
-        <v>CHUPETE</v>
+        <v>REGIO</v>
       </c>
     </row>
     <row r="182">
@@ -2951,94 +2951,94 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C182" t="str">
-        <v>El máximo goleador en la historia de Rayados es Rogelio Funes ___</v>
+        <v>Monterrey es la capital del estado de Nuevo ___</v>
       </c>
       <c r="D182" t="str">
-        <v>MORI</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B183" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C183" t="str">
-        <v>Al ídolo regiomontano Jesús Arellano le decían «El ___»</v>
+        <v>El equipo del Tec de Monterrey se llama Borregos ___</v>
       </c>
       <c r="D183" t="str">
-        <v>CABRITO</v>
+        <v>SALVAJES</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B184" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C184" t="str">
-        <v>En 2025 llegó a Rayados el famoso defensa español Sergio ___</v>
+        <v>Los Borregos juegan futbol ___</v>
       </c>
       <c r="D184" t="str">
-        <v>RAMOS</v>
+        <v>AMERICANO</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B185" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C185" t="str">
-        <v>Rayados quedó en tercer lugar del Mundial de ___ en 2012 y en 2019</v>
+        <v>Borregos es el equipo del Tecnológico de ___</v>
       </c>
       <c r="D185" t="str">
-        <v>CLUBES</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B186" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C186" t="str">
-        <v>A la barra de Rayados se le conoce como La ___</v>
+        <v>El Tec de Monterrey lo fundó el empresario Eugenio Garza ___</v>
       </c>
       <c r="D186" t="str">
-        <v>ADICCIÓN</v>
+        <v>SADA</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B187" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C187" t="str">
-        <v>El partido entre Rayados y Tigres se llama el Clásico ___</v>
+        <v>¿En qué año se fundó el Tec de Monterrey?</v>
       </c>
       <c r="D187" t="str">
-        <v>REGIO</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>RAYADOS</v>
+        <v>BORREGOS</v>
       </c>
       <c r="B188" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C188" t="str">
-        <v>Monterrey es la capital del estado de Nuevo ___</v>
+        <v>Los colores de Borregos son el azul y el ___</v>
       </c>
       <c r="D188" t="str">
-        <v>LEÓN</v>
+        <v>BLANCO</v>
       </c>
     </row>
     <row r="189">
@@ -3049,10 +3049,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C189" t="str">
-        <v>El equipo del Tec de Monterrey se llama Borregos ___</v>
+        <v>¿En qué año se inauguró el Estadio Borregos?</v>
       </c>
       <c r="D189" t="str">
-        <v>SALVAJES</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="190">
@@ -3063,10 +3063,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C190" t="str">
-        <v>Los Borregos juegan futbol ___</v>
+        <v>El Estadio Borregos se construyó en el lugar del antiguo Estadio ___</v>
       </c>
       <c r="D190" t="str">
-        <v>AMERICANO</v>
+        <v>TECNOLÓGICO</v>
       </c>
     </row>
     <row r="191">
@@ -3077,10 +3077,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C191" t="str">
-        <v>Borregos es el equipo del Tecnológico de ___</v>
+        <v>¿Qué equipo de futbol soccer jugó en el Estadio Tecnológico hasta 2015?</v>
       </c>
       <c r="D191" t="str">
-        <v>MONTERREY</v>
+        <v>RAYADOS</v>
       </c>
     </row>
     <row r="192">
@@ -3091,10 +3091,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C192" t="str">
-        <v>El Tec de Monterrey lo fundó el empresario Eugenio Garza ___</v>
+        <v>¿Cómo se llama la liga universitaria de futbol americano donde juega Borregos?</v>
       </c>
       <c r="D192" t="str">
-        <v>SADA</v>
+        <v>ONEFA</v>
       </c>
     </row>
     <row r="193">
@@ -3105,10 +3105,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C193" t="str">
-        <v>¿En qué año se fundó el Tec de Monterrey?</v>
+        <v>El gran rival universitario de Borregos son los Auténticos ___</v>
       </c>
       <c r="D193" t="str">
-        <v>1943</v>
+        <v>TIGRES</v>
       </c>
     </row>
     <row r="194">
@@ -3119,10 +3119,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C194" t="str">
-        <v>Los colores de Borregos son el azul y el ___</v>
+        <v>El legendario coach de Borregos Monterrey fue Frank ___</v>
       </c>
       <c r="D194" t="str">
-        <v>BLANCO</v>
+        <v>GONZÁLEZ</v>
       </c>
     </row>
     <row r="195">
@@ -3133,10 +3133,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C195" t="str">
-        <v>¿En qué año se inauguró el Estadio Borregos?</v>
+        <v>¿Qué animal es la mascota del Tec de Monterrey?</v>
       </c>
       <c r="D195" t="str">
-        <v>2019</v>
+        <v>BORREGO</v>
       </c>
     </row>
     <row r="196">
@@ -3147,10 +3147,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C196" t="str">
-        <v>El Estadio Borregos se construyó en el lugar del antiguo Estadio ___</v>
+        <v>Llevar el balón hasta la zona de anotación es un ___</v>
       </c>
       <c r="D196" t="str">
-        <v>TECNOLÓGICO</v>
+        <v>TOUCHDOWN</v>
       </c>
     </row>
     <row r="197">
@@ -3161,10 +3161,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C197" t="str">
-        <v>¿Qué equipo de futbol soccer jugó en el Estadio Tecnológico hasta 2015?</v>
+        <v>¿Cuántos puntos vale un touchdown?</v>
       </c>
       <c r="D197" t="str">
-        <v>RAYADOS</v>
+        <v>SEIS</v>
       </c>
     </row>
     <row r="198">
@@ -3175,10 +3175,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C198" t="str">
-        <v>¿Cómo se llama la liga universitaria de futbol americano donde juega Borregos?</v>
+        <v>¿Cuántos puntos vale un gol de campo?</v>
       </c>
       <c r="D198" t="str">
-        <v>ONEFA</v>
+        <v>TRES</v>
       </c>
     </row>
     <row r="199">
@@ -3189,10 +3189,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C199" t="str">
-        <v>El gran rival universitario de Borregos son los Auténticos ___</v>
+        <v>¿Cuántos puntos vale un safety?</v>
       </c>
       <c r="D199" t="str">
-        <v>TIGRES</v>
+        <v>DOS</v>
       </c>
     </row>
     <row r="200">
@@ -3203,10 +3203,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C200" t="str">
-        <v>El legendario coach de Borregos Monterrey fue Frank ___</v>
+        <v>Después de un touchdown se patea para ganar el punto ___</v>
       </c>
       <c r="D200" t="str">
-        <v>GONZÁLEZ</v>
+        <v>EXTRA</v>
       </c>
     </row>
     <row r="201">
@@ -3217,10 +3217,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C201" t="str">
-        <v>¿Qué animal es la mascota del Tec de Monterrey?</v>
+        <v>El jugador que lanza los pases es el mariscal de ___</v>
       </c>
       <c r="D201" t="str">
-        <v>BORREGO</v>
+        <v>CAMPO</v>
       </c>
     </row>
     <row r="202">
@@ -3231,10 +3231,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C202" t="str">
-        <v>Llevar el balón hasta la zona de anotación es un ___</v>
+        <v>¿Cuántos jugadores tiene cada equipo en la cancha?</v>
       </c>
       <c r="D202" t="str">
-        <v>TOUCHDOWN</v>
+        <v>ONCE</v>
       </c>
     </row>
     <row r="203">
@@ -3245,10 +3245,10 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C203" t="str">
-        <v>¿Cuántos puntos vale un touchdown?</v>
+        <v>¿En cuántas oportunidades hay que avanzar diez yardas?</v>
       </c>
       <c r="D203" t="str">
-        <v>SEIS</v>
+        <v>CUATRO</v>
       </c>
     </row>
     <row r="204">
@@ -3259,100 +3259,16 @@
         <v>PREGUNTA</v>
       </c>
       <c r="C204" t="str">
-        <v>¿Cuántos puntos vale un gol de campo?</v>
+        <v>La gran final de la NFL se llama el Super ___</v>
       </c>
       <c r="D204" t="str">
-        <v>TRES</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B205" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C205" t="str">
-        <v>¿Cuántos puntos vale un safety?</v>
-      </c>
-      <c r="D205" t="str">
-        <v>DOS</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B206" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C206" t="str">
-        <v>Después de un touchdown se patea para ganar el punto ___</v>
-      </c>
-      <c r="D206" t="str">
-        <v>EXTRA</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B207" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C207" t="str">
-        <v>El jugador que lanza los pases es el mariscal de ___</v>
-      </c>
-      <c r="D207" t="str">
-        <v>CAMPO</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B208" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C208" t="str">
-        <v>¿Cuántos jugadores tiene cada equipo en la cancha?</v>
-      </c>
-      <c r="D208" t="str">
-        <v>ONCE</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B209" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C209" t="str">
-        <v>¿En cuántas oportunidades hay que avanzar diez yardas?</v>
-      </c>
-      <c r="D209" t="str">
-        <v>CUATRO</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="str">
-        <v>BORREGOS</v>
-      </c>
-      <c r="B210" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C210" t="str">
-        <v>La gran final de la NFL se llama el Super ___</v>
-      </c>
-      <c r="D210" t="str">
         <v>BOWL</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D210"/>
+  <autoFilter ref="A1:D204"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D210"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D204"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ninguna pregunta se salta sin jugador; banco ampliado a 230 preguntas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/preguntas.xlsx
+++ b/datos/preguntas.xlsx
@@ -7,7 +7,7 @@
     <sheet name="INSTRUCCIONES" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'PREGUNTAS'!A1:D204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'PREGUNTAS'!A1:D231</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D231"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -929,170 +929,170 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B38" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C38" t="str">
-        <v>Corazón ___</v>
+        <v>¿Cómo se apellida Adam, el vocalista de Maroon 5?</v>
       </c>
       <c r="D38" t="str">
-        <v>PARTÍO</v>
+        <v>LEVINE</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B39" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C39" t="str">
-        <v>Amiga ___</v>
+        <v>«Moves Like Jagger» la grabaron con la cantante Christina ___</v>
       </c>
       <c r="D39" t="str">
-        <v>MÍA</v>
+        <v>AGUILERA</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B40" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C40" t="str">
-        <v>Y si fuera ___</v>
+        <v>«What Lovers Do» la grabaron con la cantante estadounidense ___</v>
       </c>
       <c r="D40" t="str">
-        <v>ELLA</v>
+        <v>SZA</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B41" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C41" t="str">
-        <v>Mi soledad y ___</v>
+        <v>«Don't Wanna Know» la grabaron con el rapero Kendrick ___</v>
       </c>
       <c r="D41" t="str">
-        <v>YO</v>
+        <v>LAMAR</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B42" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C42" t="str">
-        <v>Cuando nadie me ___</v>
+        <v>«Beautiful Mistakes» la grabaron con la rapera Megan Thee ___</v>
       </c>
       <c r="D42" t="str">
-        <v>VE</v>
+        <v>STALLION</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B43" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C43" t="str">
-        <v>Pisando ___</v>
+        <v>La melodía de «Memories» está inspirada en el famoso «Canon» del compositor ___</v>
       </c>
       <c r="D43" t="str">
-        <v>FUERTE</v>
+        <v>PACHELBEL</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B44" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C44" t="str">
-        <v>Los dos cogidos de la ___</v>
+        <v>En el video de «Animals», Adam Levine interpreta a un ___ obsesionado</v>
       </c>
       <c r="D44" t="str">
-        <v>MANO</v>
+        <v>CARNICERO</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B45" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C45" t="str">
-        <v>Deja que te ___</v>
+        <v>Adam Levine está casado con la modelo namibia Behati ___</v>
       </c>
       <c r="D45" t="str">
-        <v>BESE</v>
+        <v>PRINSLOO</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B46" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C46" t="str">
-        <v>Hoy llueve, hoy ___</v>
+        <v>Adam Levine actuó en la película de 2013 «Begin ___»</v>
       </c>
       <c r="D46" t="str">
-        <v>DUELE</v>
+        <v>AGAIN</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B47" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C47" t="str">
-        <v>No me ___</v>
+        <v>La canción de Adam Levine nominada al Óscar por «Begin Again» se llama «Lost ___»</v>
       </c>
       <c r="D47" t="str">
-        <v>COMPARES</v>
+        <v>STARS</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B48" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C48" t="str">
-        <v>Mi persona ___</v>
+        <v>En 2005 Maroon 5 ganó el Grammy a Mejor Artista ___</v>
       </c>
       <c r="D48" t="str">
-        <v>FAVORITA</v>
+        <v>NUEVO</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ALEJANDRO SANZ</v>
+        <v>MAROON 5</v>
       </c>
       <c r="B49" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C49" t="str">
-        <v>Looking for ___</v>
+        <v>Maroon 5 tuvo una residencia de conciertos en la ciudad de Las ___</v>
       </c>
       <c r="D49" t="str">
-        <v>PARADISE</v>
+        <v>VEGAS</v>
       </c>
     </row>
     <row r="50">
@@ -1103,10 +1103,10 @@
         <v>CANCION</v>
       </c>
       <c r="C50" t="str">
-        <v>Siempre es de ___</v>
+        <v>Corazón ___</v>
       </c>
       <c r="D50" t="str">
-        <v>NOCHE</v>
+        <v>PARTÍO</v>
       </c>
     </row>
     <row r="51">
@@ -1117,10 +1117,10 @@
         <v>CANCION</v>
       </c>
       <c r="C51" t="str">
-        <v>Quisiera ___</v>
+        <v>Amiga ___</v>
       </c>
       <c r="D51" t="str">
-        <v>SER</v>
+        <v>MÍA</v>
       </c>
     </row>
     <row r="52">
@@ -1131,10 +1131,10 @@
         <v>CANCION</v>
       </c>
       <c r="C52" t="str">
-        <v>Desde ___</v>
+        <v>Y si fuera ___</v>
       </c>
       <c r="D52" t="str">
-        <v>CUÁNDO</v>
+        <v>ELLA</v>
       </c>
     </row>
     <row r="53">
@@ -1145,10 +1145,10 @@
         <v>CANCION</v>
       </c>
       <c r="C53" t="str">
-        <v>Si hay ___</v>
+        <v>Mi soledad y ___</v>
       </c>
       <c r="D53" t="str">
-        <v>DIOS</v>
+        <v>YO</v>
       </c>
     </row>
     <row r="54">
@@ -1159,10 +1159,10 @@
         <v>CANCION</v>
       </c>
       <c r="C54" t="str">
-        <v>Te lo agradezco, pero ___</v>
+        <v>Cuando nadie me ___</v>
       </c>
       <c r="D54" t="str">
-        <v>NO</v>
+        <v>VE</v>
       </c>
     </row>
     <row r="55">
@@ -1170,13 +1170,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B55" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C55" t="str">
-        <v>El alma al ___</v>
+        <v>Pisando ___</v>
       </c>
       <c r="D55" t="str">
-        <v>AIRE</v>
+        <v>FUERTE</v>
       </c>
     </row>
     <row r="56">
@@ -1184,13 +1184,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B56" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C56" t="str">
-        <v>No es lo ___</v>
+        <v>Los dos cogidos de la ___</v>
       </c>
       <c r="D56" t="str">
-        <v>MISMO</v>
+        <v>MANO</v>
       </c>
     </row>
     <row r="57">
@@ -1198,13 +1198,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B57" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C57" t="str">
-        <v>Viviendo ___</v>
+        <v>Deja que te ___</v>
       </c>
       <c r="D57" t="str">
-        <v>DEPRISA</v>
+        <v>BESE</v>
       </c>
     </row>
     <row r="58">
@@ -1212,13 +1212,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B58" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C58" t="str">
-        <v>El tren de los ___</v>
+        <v>Hoy llueve, hoy ___</v>
       </c>
       <c r="D58" t="str">
-        <v>MOMENTOS</v>
+        <v>DUELE</v>
       </c>
     </row>
     <row r="59">
@@ -1226,13 +1226,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B59" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C59" t="str">
-        <v>La música no se ___</v>
+        <v>No me ___</v>
       </c>
       <c r="D59" t="str">
-        <v>TOCA</v>
+        <v>COMPARES</v>
       </c>
     </row>
     <row r="60">
@@ -1240,13 +1240,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B60" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C60" t="str">
-        <v>Paraíso ___</v>
+        <v>Mi persona ___</v>
       </c>
       <c r="D60" t="str">
-        <v>EXPRESS</v>
+        <v>FAVORITA</v>
       </c>
     </row>
     <row r="61">
@@ -1254,13 +1254,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B61" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C61" t="str">
-        <v>Si tú me ___</v>
+        <v>Looking for ___</v>
       </c>
       <c r="D61" t="str">
-        <v>MIRAS</v>
+        <v>PARADISE</v>
       </c>
     </row>
     <row r="62">
@@ -1268,13 +1268,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B62" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C62" t="str">
-        <v>¿Cómo se llama su disco de 1997, el de «Corazón partío»?</v>
+        <v>Siempre es de ___</v>
       </c>
       <c r="D62" t="str">
-        <v>MÁS</v>
+        <v>NOCHE</v>
       </c>
     </row>
     <row r="63">
@@ -1282,13 +1282,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B63" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C63" t="str">
-        <v>Su disco de 2015 se llama como un jarabe dulce: ___</v>
+        <v>Quisiera ___</v>
       </c>
       <c r="D63" t="str">
-        <v>SIROPE</v>
+        <v>SER</v>
       </c>
     </row>
     <row r="64">
@@ -1296,13 +1296,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B64" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C64" t="str">
-        <v>Su disco de 2019 tiene nombre de hashtag: #El___</v>
+        <v>Desde ___</v>
       </c>
       <c r="D64" t="str">
-        <v>DISCO</v>
+        <v>CUÁNDO</v>
       </c>
     </row>
     <row r="65">
@@ -1310,13 +1310,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B65" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C65" t="str">
-        <v>La canción que grabó con Shakira en 2005 se llama La ___</v>
+        <v>Si hay ___</v>
       </c>
       <c r="D65" t="str">
-        <v>TORTURA</v>
+        <v>DIOS</v>
       </c>
     </row>
     <row r="66">
@@ -1324,13 +1324,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B66" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C66" t="str">
-        <v>«Mi persona favorita» la grabó con la cantante Camila ___</v>
+        <v>Te lo agradezco, pero ___</v>
       </c>
       <c r="D66" t="str">
-        <v>CABELLO</v>
+        <v>NO</v>
       </c>
     </row>
     <row r="67">
@@ -1338,13 +1338,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B67" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C67" t="str">
-        <v>«Looking for Paradise» la grabó con la cantante Alicia ___</v>
+        <v>El alma al ___</v>
       </c>
       <c r="D67" t="str">
-        <v>KEYS</v>
+        <v>AIRE</v>
       </c>
     </row>
     <row r="68">
@@ -1352,13 +1352,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B68" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C68" t="str">
-        <v>«Deja que te bese» la grabó con el cantante Marc ___</v>
+        <v>No es lo ___</v>
       </c>
       <c r="D68" t="str">
-        <v>ANTHONY</v>
+        <v>MISMO</v>
       </c>
     </row>
     <row r="69">
@@ -1366,13 +1366,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B69" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C69" t="str">
-        <v>¿En qué ciudad nació el cantante?</v>
+        <v>Viviendo ___</v>
       </c>
       <c r="D69" t="str">
-        <v>MADRID</v>
+        <v>DEPRISA</v>
       </c>
     </row>
     <row r="70">
@@ -1380,13 +1380,13 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B70" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C70" t="str">
-        <v>¿De qué país es el cantante?</v>
+        <v>El tren de los ___</v>
       </c>
       <c r="D70" t="str">
-        <v>ESPAÑA</v>
+        <v>MOMENTOS</v>
       </c>
     </row>
     <row r="71">
@@ -1394,587 +1394,587 @@
         <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B71" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C71" t="str">
-        <v>¿Qué género musical andaluz se escucha en muchas de sus canciones?</v>
+        <v>La música no se ___</v>
       </c>
       <c r="D71" t="str">
-        <v>FLAMENCO</v>
+        <v>TOCA</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B72" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C72" t="str">
-        <v>¿Y todo para ___?</v>
+        <v>Paraíso ___</v>
       </c>
       <c r="D72" t="str">
-        <v>QUÉ</v>
+        <v>EXPRESS</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B73" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C73" t="str">
-        <v>Enséñame a ___</v>
+        <v>Si tú me ___</v>
       </c>
       <c r="D73" t="str">
-        <v>OLVIDAR</v>
+        <v>MIRAS</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B74" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C74" t="str">
-        <v>Alguien te va a hacer ___</v>
+        <v>¿Cómo se llama su disco de 1997, el de «Corazón partío»?</v>
       </c>
       <c r="D74" t="str">
-        <v>LLORAR</v>
+        <v>MÁS</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B75" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C75" t="str">
-        <v>¿Dónde ___?</v>
+        <v>Su disco de 2015 se llama como un jarabe dulce: ___</v>
       </c>
       <c r="D75" t="str">
-        <v>ESTÁS</v>
+        <v>SIROPE</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B76" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C76" t="str">
-        <v>Fuerte no ___</v>
+        <v>Su disco de 2019 tiene nombre de hashtag: #El___</v>
       </c>
       <c r="D76" t="str">
-        <v>SOY</v>
+        <v>DISCO</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B77" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C77" t="str">
-        <v>Nuestro destino estaba ___</v>
+        <v>La canción que grabó con Shakira en 2005 se llama La ___</v>
       </c>
       <c r="D77" t="str">
-        <v>ESCRITO</v>
+        <v>TORTURA</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B78" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C78" t="str">
-        <v>¿Qué instrumento toca el vocalista del grupo mientras canta?</v>
+        <v>«Mi persona favorita» la grabó con la cantante Camila ___</v>
       </c>
       <c r="D78" t="str">
-        <v>ACORDEÓN</v>
+        <v>CABELLO</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B79" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C79" t="str">
-        <v>¿De qué estado de Estados Unidos es el grupo?</v>
+        <v>«Looking for Paradise» la grabó con la cantante Alicia ___</v>
       </c>
       <c r="D79" t="str">
-        <v>TEXAS</v>
+        <v>KEYS</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B80" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C80" t="str">
-        <v>¿En qué pueblo de Texas nació el grupo?</v>
+        <v>«Deja que te bese» la grabó con el cantante Marc ___</v>
       </c>
       <c r="D80" t="str">
-        <v>ZAPATA</v>
+        <v>ANTHONY</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B81" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C81" t="str">
-        <v>La guitarra de doce cuerdas típica del norteño se llama bajo ___</v>
+        <v>¿En qué ciudad nació el cantante?</v>
       </c>
       <c r="D81" t="str">
-        <v>SEXTO</v>
+        <v>MADRID</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>INTOCABLE</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B82" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C82" t="str">
-        <v>¿Cómo se llama la música de los mexicanos de Texas que toca el grupo?</v>
+        <v>¿De qué país es el cantante?</v>
       </c>
       <c r="D82" t="str">
-        <v>TEJANO</v>
+        <v>ESPAÑA</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B83" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C83" t="str">
-        <v>Al acordeonista Ramón Ayala le dicen el Rey del ___</v>
+        <v>¿Qué género musical andaluz se escucha en muchas de sus canciones?</v>
       </c>
       <c r="D83" t="str">
-        <v>ACORDEÓN</v>
+        <v>FLAMENCO</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B84" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C84" t="str">
-        <v>«Tragos amargos» es un clásico de Ramón ___</v>
+        <v>Su disco de 2021 lleva su apellido artístico: ___</v>
       </c>
       <c r="D84" t="str">
-        <v>AYALA</v>
+        <v>SANZ</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B85" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C85" t="str">
-        <v>«La puerta negra» es de Los Tigres del ___</v>
+        <v>El nombre real de Alejandro Sanz es Alejandro Sánchez ___</v>
       </c>
       <c r="D85" t="str">
-        <v>NORTE</v>
+        <v>PIZARRO</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B86" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C86" t="str">
-        <v>«Contrabando y traición» es de Los Tigres del ___</v>
+        <v>Alejandro Sanz es el artista español con más premios ___</v>
       </c>
       <c r="D86" t="str">
-        <v>NORTE</v>
+        <v>GRAMMY</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B87" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C87" t="str">
-        <v>«Me caí de la nube» es un clásico de Cornelio ___</v>
+        <v>¿Con qué cantante colombiana grabó «La tortura»?</v>
       </c>
       <c r="D87" t="str">
-        <v>REYNA</v>
+        <v>SHAKIRA</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B88" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C88" t="str">
-        <v>«Laurita Garza» es de Los Invasores de Nuevo ___</v>
+        <v>Regálame la silla donde te ___</v>
       </c>
       <c r="D88" t="str">
-        <v>LEÓN</v>
+        <v>ESPERÉ</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B89" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C89" t="str">
-        <v>Ramón Ayala y Cornelio Reyna formaron Los Relámpagos del ___</v>
+        <v>Llamando a la mujer ___</v>
       </c>
       <c r="D89" t="str">
-        <v>NORTE</v>
+        <v>ARAÑA</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>NORTEÑO</v>
+        <v>ALEJANDRO SANZ</v>
       </c>
       <c r="B90" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C90" t="str">
-        <v>¿Cómo le dicen a Selena? La reina del Tex-___</v>
+        <v>A la primera ___</v>
       </c>
       <c r="D90" t="str">
-        <v>MEX</v>
+        <v>PERSONA</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>NORTEÑO</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B91" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C91" t="str">
-        <v>¿Qué baile europeo, de ritmo rápido, está en las raíces del norteño?</v>
+        <v>¿Y todo para ___?</v>
       </c>
       <c r="D91" t="str">
-        <v>POLKA</v>
+        <v>QUÉ</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>NORTEÑO</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B92" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C92" t="str">
-        <v>¿De qué ciudad es el grupo norteño Pesado?</v>
+        <v>Enséñame a ___</v>
       </c>
       <c r="D92" t="str">
-        <v>MONTERREY</v>
+        <v>OLVIDAR</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B93" t="str">
         <v>CANCION</v>
       </c>
       <c r="C93" t="str">
-        <v>Da Ya Think I'm ___?</v>
+        <v>Alguien te va a hacer ___</v>
       </c>
       <c r="D93" t="str">
-        <v>SEXY</v>
+        <v>LLORAR</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B94" t="str">
         <v>CANCION</v>
       </c>
       <c r="C94" t="str">
-        <v>Maggie ___</v>
+        <v>¿Dónde ___?</v>
       </c>
       <c r="D94" t="str">
-        <v>MAY</v>
+        <v>ESTÁS</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B95" t="str">
         <v>CANCION</v>
       </c>
       <c r="C95" t="str">
-        <v>Young ___</v>
+        <v>Fuerte no ___</v>
       </c>
       <c r="D95" t="str">
-        <v>TURKS</v>
+        <v>SOY</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B96" t="str">
-        <v>CANCION</v>
+        <v>DISCO</v>
       </c>
       <c r="C96" t="str">
-        <v>Have I Told You ___</v>
+        <v>Nuestro destino estaba ___</v>
       </c>
       <c r="D96" t="str">
-        <v>LATELY</v>
+        <v>ESCRITO</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B97" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C97" t="str">
-        <v>Forever ___</v>
+        <v>¿Qué instrumento toca el vocalista del grupo mientras canta?</v>
       </c>
       <c r="D97" t="str">
-        <v>YOUNG</v>
+        <v>ACORDEÓN</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B98" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C98" t="str">
-        <v>Some Guys Have All the ___</v>
+        <v>¿De qué estado de Estados Unidos es el grupo?</v>
       </c>
       <c r="D98" t="str">
-        <v>LUCK</v>
+        <v>TEXAS</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B99" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C99" t="str">
-        <v>Hot ___</v>
+        <v>¿En qué pueblo de Texas nació el grupo?</v>
       </c>
       <c r="D99" t="str">
-        <v>LEGS</v>
+        <v>ZAPATA</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B100" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C100" t="str">
-        <v>Tonight's the ___</v>
+        <v>La guitarra de doce cuerdas típica del norteño se llama bajo ___</v>
       </c>
       <c r="D100" t="str">
-        <v>NIGHT</v>
+        <v>SEXTO</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B101" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C101" t="str">
-        <v>Baby ___</v>
+        <v>¿Cómo se llama la música de los mexicanos de Texas que toca el grupo?</v>
       </c>
       <c r="D101" t="str">
-        <v>JANE</v>
+        <v>TEJANO</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>ROD STEWART</v>
+        <v>INTOCABLE</v>
       </c>
       <c r="B102" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C102" t="str">
-        <v>Downtown ___</v>
+        <v>¿Cómo se apellida Ricky, el vocalista y acordeonista de Intocable?</v>
       </c>
       <c r="D102" t="str">
-        <v>TRAIN</v>
+        <v>MUÑOZ</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B103" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C103" t="str">
-        <v>Rhythm of My ___</v>
+        <v>Al acordeonista Ramón Ayala le dicen el Rey del ___</v>
       </c>
       <c r="D103" t="str">
-        <v>HEART</v>
+        <v>ACORDEÓN</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B104" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C104" t="str">
-        <v>The First ___ Is the Deepest</v>
+        <v>«Tragos amargos» es un clásico de Ramón ___</v>
       </c>
       <c r="D104" t="str">
-        <v>CUT</v>
+        <v>AYALA</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B105" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C105" t="str">
-        <v>You Wear It ___</v>
+        <v>«La puerta negra» es de Los Tigres del ___</v>
       </c>
       <c r="D105" t="str">
-        <v>WELL</v>
+        <v>NORTE</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B106" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C106" t="str">
-        <v>I Don't Want to Talk About ___</v>
+        <v>«Contrabando y traición» es de Los Tigres del ___</v>
       </c>
       <c r="D106" t="str">
-        <v>IT</v>
+        <v>NORTE</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B107" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C107" t="str">
-        <v>Reason to ___</v>
+        <v>«Me caí de la nube» es un clásico de Cornelio ___</v>
       </c>
       <c r="D107" t="str">
-        <v>BELIEVE</v>
+        <v>REYNA</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B108" t="str">
-        <v>CANCION</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C108" t="str">
-        <v>All for ___</v>
+        <v>«Laurita Garza» es de Los Invasores de Nuevo ___</v>
       </c>
       <c r="D108" t="str">
-        <v>LOVE</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B109" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C109" t="str">
-        <v>Every Picture Tells a ___</v>
+        <v>Ramón Ayala y Cornelio Reyna formaron Los Relámpagos del ___</v>
       </c>
       <c r="D109" t="str">
-        <v>STORY</v>
+        <v>NORTE</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B110" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C110" t="str">
-        <v>Atlantic ___</v>
+        <v>¿Cómo le dicen a Selena? La reina del Tex-___</v>
       </c>
       <c r="D110" t="str">
-        <v>CROSSING</v>
+        <v>MEX</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B111" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C111" t="str">
-        <v>Blondes Have More ___</v>
+        <v>¿Qué baile europeo, de ritmo rápido, está en las raíces del norteño?</v>
       </c>
       <c r="D111" t="str">
-        <v>FUN</v>
+        <v>POLKA</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>ROD STEWART</v>
+        <v>NORTEÑO</v>
       </c>
       <c r="B112" t="str">
-        <v>DISCO</v>
+        <v>PREGUNTA</v>
       </c>
       <c r="C112" t="str">
-        <v>A Night on the ___</v>
+        <v>¿De qué ciudad es el grupo norteño Pesado?</v>
       </c>
       <c r="D112" t="str">
-        <v>TOWN</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="113">
@@ -1982,13 +1982,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B113" t="str">
-        <v>DISCO</v>
+        <v>CANCION</v>
       </c>
       <c r="C113" t="str">
-        <v>Gasoline ___</v>
+        <v>Da Ya Think I'm ___?</v>
       </c>
       <c r="D113" t="str">
-        <v>ALLEY</v>
+        <v>SEXY</v>
       </c>
     </row>
     <row r="114">
@@ -1996,13 +1996,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B114" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C114" t="str">
-        <v>¿Qué canción de 1975 habla de navegar por el mar?</v>
+        <v>Maggie ___</v>
       </c>
       <c r="D114" t="str">
-        <v>SAILING</v>
+        <v>MAY</v>
       </c>
     </row>
     <row r="115">
@@ -2010,13 +2010,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B115" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C115" t="str">
-        <v>Antes de ser solista, cantó en la banda The ___</v>
+        <v>Young ___</v>
       </c>
       <c r="D115" t="str">
-        <v>FACES</v>
+        <v>TURKS</v>
       </c>
     </row>
     <row r="116">
@@ -2024,13 +2024,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B116" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C116" t="str">
-        <v>Su primer grupo famoso lo formó con el guitarrista Jeff ___</v>
+        <v>Have I Told You ___</v>
       </c>
       <c r="D116" t="str">
-        <v>BECK</v>
+        <v>LATELY</v>
       </c>
     </row>
     <row r="117">
@@ -2038,13 +2038,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B117" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C117" t="str">
-        <v>En los años 60 lo apodaban «Rod the ___»</v>
+        <v>Forever ___</v>
       </c>
       <c r="D117" t="str">
-        <v>MOD</v>
+        <v>YOUNG</v>
       </c>
     </row>
     <row r="118">
@@ -2052,13 +2052,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B118" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C118" t="str">
-        <v>¿En qué ciudad nació el cantante?</v>
+        <v>Some Guys Have All the ___</v>
       </c>
       <c r="D118" t="str">
-        <v>LONDRES</v>
+        <v>LUCK</v>
       </c>
     </row>
     <row r="119">
@@ -2066,13 +2066,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B119" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C119" t="str">
-        <v>¿De qué país es su familia paterna, al que siempre dice pertenecer?</v>
+        <v>Hot ___</v>
       </c>
       <c r="D119" t="str">
-        <v>ESCOCIA</v>
+        <v>LEGS</v>
       </c>
     </row>
     <row r="120">
@@ -2080,13 +2080,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B120" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C120" t="str">
-        <v>¿De qué equipo de futbol escocés es fanático el cantante?</v>
+        <v>Tonight's the ___</v>
       </c>
       <c r="D120" t="str">
-        <v>CELTIC</v>
+        <v>NIGHT</v>
       </c>
     </row>
     <row r="121">
@@ -2094,13 +2094,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B121" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C121" t="str">
-        <v>Su serie de discos de clásicos se llama The Great American ___</v>
+        <v>Baby ___</v>
       </c>
       <c r="D121" t="str">
-        <v>SONGBOOK</v>
+        <v>JANE</v>
       </c>
     </row>
     <row r="122">
@@ -2108,13 +2108,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B122" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C122" t="str">
-        <v>Desde 2016 es caballero británico, así que antes de su nombre lleva el título de ___</v>
+        <v>Downtown ___</v>
       </c>
       <c r="D122" t="str">
-        <v>SIR</v>
+        <v>TRAIN</v>
       </c>
     </row>
     <row r="123">
@@ -2122,13 +2122,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B123" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C123" t="str">
-        <v>«All for Love» la grabó con Bryan Adams y ___</v>
+        <v>Rhythm of My ___</v>
       </c>
       <c r="D123" t="str">
-        <v>STING</v>
+        <v>HEART</v>
       </c>
     </row>
     <row r="124">
@@ -2136,13 +2136,13 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B124" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C124" t="str">
-        <v>¿En qué playa de Río de Janeiro dio un concierto histórico en 1994?</v>
+        <v>The First ___ Is the Deepest</v>
       </c>
       <c r="D124" t="str">
-        <v>COPACABANA</v>
+        <v>CUT</v>
       </c>
     </row>
     <row r="125">
@@ -2150,1125 +2150,1503 @@
         <v>ROD STEWART</v>
       </c>
       <c r="B125" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C125" t="str">
-        <v>Su gran pasatiempo es armar maquetas gigantes de ___</v>
+        <v>You Wear It ___</v>
       </c>
       <c r="D125" t="str">
-        <v>TRENES</v>
+        <v>WELL</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B126" t="str">
         <v>CANCION</v>
       </c>
       <c r="C126" t="str">
-        <v>Ella quiere ___</v>
+        <v>I Don't Want to Talk About ___</v>
       </c>
       <c r="D126" t="str">
-        <v>BEBER</v>
+        <v>IT</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B127" t="str">
         <v>CANCION</v>
       </c>
       <c r="C127" t="str">
-        <v>Hasta que Dios ___</v>
+        <v>Reason to ___</v>
       </c>
       <c r="D127" t="str">
-        <v>DIGA</v>
+        <v>BELIEVE</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B128" t="str">
         <v>CANCION</v>
       </c>
       <c r="C128" t="str">
-        <v>Mejor que ___</v>
+        <v>All for ___</v>
       </c>
       <c r="D128" t="str">
-        <v>YO</v>
+        <v>LOVE</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B129" t="str">
         <v>DISCO</v>
       </c>
       <c r="C129" t="str">
-        <v>Las leyendas nunca ___</v>
+        <v>Every Picture Tells a ___</v>
       </c>
       <c r="D129" t="str">
-        <v>MUEREN</v>
+        <v>STORY</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B130" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C130" t="str">
-        <v>Su disco con Ozuna se llama Los ___</v>
+        <v>Atlantic ___</v>
       </c>
       <c r="D130" t="str">
-        <v>DIOSES</v>
+        <v>CROSSING</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B131" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C131" t="str">
-        <v>El cantante nació en Carolina, Puerto ___</v>
+        <v>Blondes Have More ___</v>
       </c>
       <c r="D131" t="str">
-        <v>RICO</v>
+        <v>FUN</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B132" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C132" t="str">
-        <v>¿Con qué cantante puertorriqueño grabó el disco «Los Dioses»?</v>
+        <v>A Night on the ___</v>
       </c>
       <c r="D132" t="str">
-        <v>OZUNA</v>
+        <v>TOWN</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B133" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C133" t="str">
-        <v>¿Qué canción de 2019 grabó con Karol G?</v>
+        <v>Gasoline ___</v>
       </c>
       <c r="D133" t="str">
-        <v>SECRETO</v>
+        <v>ALLEY</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B134" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C134" t="str">
-        <v>¿Qué canción de 2019 grabó junto a Daddy Yankee, Karol G, Ozuna y J Balvin?</v>
+        <v>¿Qué canción de 1975 habla de navegar por el mar?</v>
       </c>
       <c r="D134" t="str">
-        <v>CHINA</v>
+        <v>SAILING</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B135" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C135" t="str">
-        <v>¿Qué canción grabó con Tekashi 6ix9ine en 2018?</v>
+        <v>Antes de ser solista, cantó en la banda The ___</v>
       </c>
       <c r="D135" t="str">
-        <v>BEBÉ</v>
+        <v>FACES</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B136" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C136" t="str">
-        <v>¿Cómo se llama su primer gran éxito, de 2016?</v>
+        <v>Su primer grupo famoso lo formó con el guitarrista Jeff ___</v>
       </c>
       <c r="D136" t="str">
-        <v>SOLA</v>
+        <v>BECK</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B137" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C137" t="str">
-        <v>El remix de «Sola» lo grabó con Daddy Yankee, Wisin, Farruko y Zion &amp; ___</v>
+        <v>En los años 60 lo apodaban «Rod the ___»</v>
       </c>
       <c r="D137" t="str">
-        <v>LENNOX</v>
+        <v>MOD</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B138" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C138" t="str">
-        <v>«Adicto» la grabó con Ozuna y el productor ___</v>
+        <v>¿En qué ciudad nació el cantante?</v>
       </c>
       <c r="D138" t="str">
-        <v>TAINY</v>
+        <v>LONDRES</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B139" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C139" t="str">
-        <v>«Hasta que Dios diga» la grabó con Bad ___</v>
+        <v>¿De qué país es su familia paterna, al que siempre dice pertenecer?</v>
       </c>
       <c r="D139" t="str">
-        <v>BUNNY</v>
+        <v>ESCOCIA</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>ANUEL AA</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B140" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C140" t="str">
-        <v>Además del reguetón, su género es el ___ latino</v>
+        <v>¿De qué equipo de futbol escocés es fanático el cantante?</v>
       </c>
       <c r="D140" t="str">
-        <v>TRAP</v>
+        <v>CELTIC</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B141" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C141" t="str">
-        <v>¿Cómo se llama el estadio de Tigres? Estadio ___</v>
+        <v>Su serie de discos de clásicos se llama The Great American ___</v>
       </c>
       <c r="D141" t="str">
-        <v>UNIVERSITARIO</v>
+        <v>SONGBOOK</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B142" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C142" t="str">
-        <v>¿Cómo le dicen al Estadio Universitario por lo caliente de su ambiente?</v>
+        <v>Desde 2016 es caballero británico, así que antes de su nombre lleva el título de ___</v>
       </c>
       <c r="D142" t="str">
-        <v>VOLCÁN</v>
+        <v>SIR</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B143" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C143" t="str">
-        <v>El Volcán está en el municipio de San Nicolás de los ___</v>
+        <v>«All for Love» la grabó con Bryan Adams y ___</v>
       </c>
       <c r="D143" t="str">
-        <v>GARZA</v>
+        <v>STING</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B144" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C144" t="str">
-        <v>Tigres es el equipo de la Universidad Autónoma de Nuevo ___</v>
+        <v>¿En qué playa de Río de Janeiro dio un concierto histórico en 1994?</v>
       </c>
       <c r="D144" t="str">
-        <v>LEÓN</v>
+        <v>COPACABANA</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B145" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C145" t="str">
-        <v>¿En qué año se fundó Tigres?</v>
+        <v>Su gran pasatiempo es armar maquetas gigantes de ___</v>
       </c>
       <c r="D145" t="str">
-        <v>1960</v>
+        <v>TRENES</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B146" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C146" t="str">
-        <v>Los colores de Tigres son el azul y el ___</v>
+        <v>Ronnie Wood, su compañero en The Faces, después entró a The Rolling ___</v>
       </c>
       <c r="D146" t="str">
-        <v>AMARILLO</v>
+        <v>STONES</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>TIGRES</v>
+        <v>ROD STEWART</v>
       </c>
       <c r="B147" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C147" t="str">
-        <v>Por su uniforme amarillo y azul, a Tigres también le dicen los ___</v>
+        <v>«Da Ya Think I'm Sexy?» (1978) tiene el ritmo de la música ___</v>
       </c>
       <c r="D147" t="str">
-        <v>AURIAZULES</v>
+        <v>DISCO</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B148" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C148" t="str">
-        <v>¿Qué animal es el emblema de la UANL?</v>
+        <v>Ella quiere ___</v>
       </c>
       <c r="D148" t="str">
-        <v>TIGRE</v>
+        <v>BEBER</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B149" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C149" t="str">
-        <v>¿Cómo se apellida André-Pierre, el máximo goleador en la historia de Tigres?</v>
+        <v>Hasta que Dios ___</v>
       </c>
       <c r="D149" t="str">
-        <v>GIGNAC</v>
+        <v>DIGA</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B150" t="str">
-        <v>PREGUNTA</v>
+        <v>CANCION</v>
       </c>
       <c r="C150" t="str">
-        <v>¿De qué país es André-Pierre Gignac?</v>
+        <v>Mejor que ___</v>
       </c>
       <c r="D150" t="str">
-        <v>FRANCIA</v>
+        <v>YO</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B151" t="str">
-        <v>PREGUNTA</v>
+        <v>DISCO</v>
       </c>
       <c r="C151" t="str">
-        <v>Con el técnico Ricardo «Tuca» ___, Tigres ganó cinco títulos de liga</v>
+        <v>Las leyendas nunca ___</v>
       </c>
       <c r="D151" t="str">
-        <v>FERRETTI</v>
+        <v>MUEREN</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B152" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C152" t="str">
-        <v>¿De qué país es el técnico Ricardo «Tuca» Ferretti?</v>
+        <v>Su disco con Ozuna se llama Los ___</v>
       </c>
       <c r="D152" t="str">
-        <v>BRASIL</v>
+        <v>DIOSES</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B153" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C153" t="str">
-        <v>Al portero argentino Nahuel Guzmán le apodan «El ___»</v>
+        <v>El cantante nació en Carolina, Puerto ___</v>
       </c>
       <c r="D153" t="str">
-        <v>PATÓN</v>
+        <v>RICO</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B154" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C154" t="str">
-        <v>El mediocampista argentino que fue capitán de Tigres: Guido ___</v>
+        <v>¿Con qué cantante puertorriqueño grabó el disco «Los Dioses»?</v>
       </c>
       <c r="D154" t="str">
-        <v>PIZARRO</v>
+        <v>OZUNA</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B155" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C155" t="str">
-        <v>En 2020 Tigres ganó la Concacaf ___ League</v>
+        <v>¿Qué canción de 2019 grabó con Karol G?</v>
       </c>
       <c r="D155" t="str">
-        <v>CHAMPIONS</v>
+        <v>SECRETO</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B156" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C156" t="str">
-        <v>En la final del Mundial de Clubes 2020, Tigres enfrentó al Bayern ___</v>
+        <v>¿Qué canción de 2019 grabó junto a Daddy Yankee, Karol G, Ozuna y J Balvin?</v>
       </c>
       <c r="D156" t="str">
-        <v>MÚNICH</v>
+        <v>CHINA</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B157" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C157" t="str">
-        <v>A la afición de Tigres se le conoce como «La afición ___»</v>
+        <v>¿Qué canción grabó con Tekashi 6ix9ine en 2018?</v>
       </c>
       <c r="D157" t="str">
-        <v>INCOMPARABLE</v>
+        <v>BEBÉ</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B158" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C158" t="str">
-        <v>La barra de Tigres se llama Libres y ___</v>
+        <v>¿Cómo se llama su primer gran éxito, de 2016?</v>
       </c>
       <c r="D158" t="str">
-        <v>LOKOS</v>
+        <v>SOLA</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B159" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C159" t="str">
-        <v>El partido entre Tigres y Rayados se llama el Clásico ___</v>
+        <v>El remix de «Sola» lo grabó con Daddy Yankee, Wisin, Farruko y Zion &amp; ___</v>
       </c>
       <c r="D159" t="str">
-        <v>REGIO</v>
+        <v>LENNOX</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>TIGRES</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B160" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C160" t="str">
-        <v>¿Cómo se llama el equipo de mujeres de la UANL? Tigres ___</v>
+        <v>«Adicto» la grabó con Ozuna y el productor ___</v>
       </c>
       <c r="D160" t="str">
-        <v>FEMENIL</v>
+        <v>TAINY</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B161" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C161" t="str">
-        <v>¿Cómo se llama el estadio de Rayados? Estadio ___</v>
+        <v>«Hasta que Dios diga» la grabó con Bad ___</v>
       </c>
       <c r="D161" t="str">
-        <v>BBVA</v>
+        <v>BUNNY</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B162" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C162" t="str">
-        <v>Al Estadio BBVA le dicen el Gigante de ___</v>
+        <v>Además del reguetón, su género es el ___ latino</v>
       </c>
       <c r="D162" t="str">
-        <v>ACERO</v>
+        <v>TRAP</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B163" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C163" t="str">
-        <v>¿En qué año se inauguró el Estadio BBVA?</v>
+        <v>¿Cómo se llama su disco de 2020, que lleva su primer nombre?</v>
       </c>
       <c r="D163" t="str">
-        <v>2015</v>
+        <v>EMMANUEL</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B164" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C164" t="str">
-        <v>¿En qué municipio está el Estadio BBVA?</v>
+        <v>El nombre real de Anuel AA es Emmanuel ___ Santiago</v>
       </c>
       <c r="D164" t="str">
-        <v>GUADALUPE</v>
+        <v>GAZMEY</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B165" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C165" t="str">
-        <v>El Estadio BBVA está junto al parque ecológico La ___</v>
+        <v>Su disco de 2024 se llama «___»</v>
       </c>
       <c r="D165" t="str">
-        <v>PASTORA</v>
+        <v>ROMPECORAZONES</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B166" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C166" t="str">
-        <v>Desde las gradas del BBVA se ve el Cerro de la ___</v>
+        <v>«China» usa parte de la melodía de «Hips Don't Lie», de ___</v>
       </c>
       <c r="D166" t="str">
-        <v>SILLA</v>
+        <v>SHAKIRA</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>RAYADOS</v>
+        <v>ANUEL AA</v>
       </c>
       <c r="B167" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C167" t="str">
-        <v>Antes del BBVA, Rayados jugaba de local en el Estadio ___</v>
+        <v>¿En qué año nació Anuel AA?</v>
       </c>
       <c r="D167" t="str">
-        <v>TECNOLÓGICO</v>
+        <v>1992</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B168" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C168" t="str">
-        <v>El nombre oficial de Rayados es Club de Futbol ___</v>
+        <v>¿Cómo se llama el estadio de Tigres? Estadio ___</v>
       </c>
       <c r="D168" t="str">
-        <v>MONTERREY</v>
+        <v>UNIVERSITARIO</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B169" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C169" t="str">
-        <v>¿En qué año se fundó Rayados?</v>
+        <v>¿Cómo le dicen al Estadio Universitario por lo caliente de su ambiente?</v>
       </c>
       <c r="D169" t="str">
-        <v>1945</v>
+        <v>VOLCÁN</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B170" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C170" t="str">
-        <v>El uniforme de Rayados tiene rayas verticales azules y ___</v>
+        <v>El Volcán está en el municipio de San Nicolás de los ___</v>
       </c>
       <c r="D170" t="str">
-        <v>BLANCAS</v>
+        <v>GARZA</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B171" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C171" t="str">
-        <v>Además de Rayados, al equipo también le dicen La ___</v>
+        <v>Tigres es el equipo de la Universidad Autónoma de Nuevo ___</v>
       </c>
       <c r="D171" t="str">
-        <v>PANDILLA</v>
+        <v>LEÓN</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B172" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C172" t="str">
-        <v>¿En qué año ganó Rayados su primer título de liga?</v>
+        <v>¿En qué año se fundó Tigres?</v>
       </c>
       <c r="D172" t="str">
-        <v>1986</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B173" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C173" t="str">
-        <v>Entre 2011 y 2013, ¿cuántas Concachampions seguidas ganó Rayados?</v>
+        <v>Los colores de Tigres son el azul y el ___</v>
       </c>
       <c r="D173" t="str">
-        <v>TRES</v>
+        <v>AMARILLO</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B174" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C174" t="str">
-        <v>Al técnico Víctor Manuel Vucetich le dicen el Rey ___</v>
+        <v>Por su uniforme amarillo y azul, a Tigres también le dicen los ___</v>
       </c>
       <c r="D174" t="str">
-        <v>MIDAS</v>
+        <v>AURIAZULES</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B175" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C175" t="str">
-        <v>Al delantero chileno Humberto Suazo le decían «___»</v>
+        <v>¿Qué animal es el emblema de la UANL?</v>
       </c>
       <c r="D175" t="str">
-        <v>CHUPETE</v>
+        <v>TIGRE</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B176" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C176" t="str">
-        <v>El máximo goleador en la historia de Rayados es Rogelio Funes ___</v>
+        <v>¿Cómo se apellida André-Pierre, el máximo goleador en la historia de Tigres?</v>
       </c>
       <c r="D176" t="str">
-        <v>MORI</v>
+        <v>GIGNAC</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B177" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C177" t="str">
-        <v>Al ídolo regiomontano Jesús Arellano le decían «El ___»</v>
+        <v>¿De qué país es André-Pierre Gignac?</v>
       </c>
       <c r="D177" t="str">
-        <v>CABRITO</v>
+        <v>FRANCIA</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B178" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C178" t="str">
-        <v>En 2025 llegó a Rayados el famoso defensa español Sergio ___</v>
+        <v>Con el técnico Ricardo «Tuca» ___, Tigres ganó cinco títulos de liga</v>
       </c>
       <c r="D178" t="str">
-        <v>RAMOS</v>
+        <v>FERRETTI</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B179" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C179" t="str">
-        <v>Rayados quedó en tercer lugar del Mundial de ___ en 2012 y en 2019</v>
+        <v>¿De qué país es el técnico Ricardo «Tuca» Ferretti?</v>
       </c>
       <c r="D179" t="str">
-        <v>CLUBES</v>
+        <v>BRASIL</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B180" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C180" t="str">
-        <v>A la barra de Rayados se le conoce como La ___</v>
+        <v>Al portero argentino Nahuel Guzmán le apodan «El ___»</v>
       </c>
       <c r="D180" t="str">
-        <v>ADICCIÓN</v>
+        <v>PATÓN</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B181" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C181" t="str">
-        <v>El partido entre Rayados y Tigres se llama el Clásico ___</v>
+        <v>El mediocampista argentino que fue capitán de Tigres: Guido ___</v>
       </c>
       <c r="D181" t="str">
-        <v>REGIO</v>
+        <v>PIZARRO</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>RAYADOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B182" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C182" t="str">
-        <v>Monterrey es la capital del estado de Nuevo ___</v>
+        <v>En 2020 Tigres ganó la Concacaf ___ League</v>
       </c>
       <c r="D182" t="str">
-        <v>LEÓN</v>
+        <v>CHAMPIONS</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>BORREGOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B183" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C183" t="str">
-        <v>El equipo del Tec de Monterrey se llama Borregos ___</v>
+        <v>En la final del Mundial de Clubes 2020, Tigres enfrentó al Bayern ___</v>
       </c>
       <c r="D183" t="str">
-        <v>SALVAJES</v>
+        <v>MÚNICH</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>BORREGOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B184" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C184" t="str">
-        <v>Los Borregos juegan futbol ___</v>
+        <v>A la afición de Tigres se le conoce como «La afición ___»</v>
       </c>
       <c r="D184" t="str">
-        <v>AMERICANO</v>
+        <v>INCOMPARABLE</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>BORREGOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B185" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C185" t="str">
-        <v>Borregos es el equipo del Tecnológico de ___</v>
+        <v>La barra de Tigres se llama Libres y ___</v>
       </c>
       <c r="D185" t="str">
-        <v>MONTERREY</v>
+        <v>LOKOS</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>BORREGOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B186" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C186" t="str">
-        <v>El Tec de Monterrey lo fundó el empresario Eugenio Garza ___</v>
+        <v>El partido entre Tigres y Rayados se llama el Clásico ___</v>
       </c>
       <c r="D186" t="str">
-        <v>SADA</v>
+        <v>REGIO</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>BORREGOS</v>
+        <v>TIGRES</v>
       </c>
       <c r="B187" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C187" t="str">
-        <v>¿En qué año se fundó el Tec de Monterrey?</v>
+        <v>¿Cómo se llama el equipo de mujeres de la UANL? Tigres ___</v>
       </c>
       <c r="D187" t="str">
-        <v>1943</v>
+        <v>FEMENIL</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B188" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C188" t="str">
-        <v>Los colores de Borregos son el azul y el ___</v>
+        <v>¿Cómo se llama el estadio de Rayados? Estadio ___</v>
       </c>
       <c r="D188" t="str">
-        <v>BLANCO</v>
+        <v>BBVA</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B189" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C189" t="str">
-        <v>¿En qué año se inauguró el Estadio Borregos?</v>
+        <v>Al Estadio BBVA le dicen el Gigante de ___</v>
       </c>
       <c r="D189" t="str">
-        <v>2019</v>
+        <v>ACERO</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B190" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C190" t="str">
-        <v>El Estadio Borregos se construyó en el lugar del antiguo Estadio ___</v>
+        <v>¿En qué año se inauguró el Estadio BBVA?</v>
       </c>
       <c r="D190" t="str">
-        <v>TECNOLÓGICO</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B191" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C191" t="str">
-        <v>¿Qué equipo de futbol soccer jugó en el Estadio Tecnológico hasta 2015?</v>
+        <v>¿En qué municipio está el Estadio BBVA?</v>
       </c>
       <c r="D191" t="str">
-        <v>RAYADOS</v>
+        <v>GUADALUPE</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B192" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C192" t="str">
-        <v>¿Cómo se llama la liga universitaria de futbol americano donde juega Borregos?</v>
+        <v>El Estadio BBVA está junto al parque ecológico La ___</v>
       </c>
       <c r="D192" t="str">
-        <v>ONEFA</v>
+        <v>PASTORA</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B193" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C193" t="str">
-        <v>El gran rival universitario de Borregos son los Auténticos ___</v>
+        <v>Desde las gradas del BBVA se ve el Cerro de la ___</v>
       </c>
       <c r="D193" t="str">
-        <v>TIGRES</v>
+        <v>SILLA</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B194" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C194" t="str">
-        <v>El legendario coach de Borregos Monterrey fue Frank ___</v>
+        <v>Antes del BBVA, Rayados jugaba de local en el Estadio ___</v>
       </c>
       <c r="D194" t="str">
-        <v>GONZÁLEZ</v>
+        <v>TECNOLÓGICO</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B195" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C195" t="str">
-        <v>¿Qué animal es la mascota del Tec de Monterrey?</v>
+        <v>El nombre oficial de Rayados es Club de Futbol ___</v>
       </c>
       <c r="D195" t="str">
-        <v>BORREGO</v>
+        <v>MONTERREY</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B196" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C196" t="str">
-        <v>Llevar el balón hasta la zona de anotación es un ___</v>
+        <v>¿En qué año se fundó Rayados?</v>
       </c>
       <c r="D196" t="str">
-        <v>TOUCHDOWN</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B197" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C197" t="str">
-        <v>¿Cuántos puntos vale un touchdown?</v>
+        <v>El uniforme de Rayados tiene rayas verticales azules y ___</v>
       </c>
       <c r="D197" t="str">
-        <v>SEIS</v>
+        <v>BLANCAS</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B198" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C198" t="str">
-        <v>¿Cuántos puntos vale un gol de campo?</v>
+        <v>Además de Rayados, al equipo también le dicen La ___</v>
       </c>
       <c r="D198" t="str">
-        <v>TRES</v>
+        <v>PANDILLA</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B199" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C199" t="str">
-        <v>¿Cuántos puntos vale un safety?</v>
+        <v>¿En qué año ganó Rayados su primer título de liga?</v>
       </c>
       <c r="D199" t="str">
-        <v>DOS</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B200" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C200" t="str">
-        <v>Después de un touchdown se patea para ganar el punto ___</v>
+        <v>Entre 2011 y 2013, ¿cuántas Concachampions seguidas ganó Rayados?</v>
       </c>
       <c r="D200" t="str">
-        <v>EXTRA</v>
+        <v>TRES</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B201" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C201" t="str">
-        <v>El jugador que lanza los pases es el mariscal de ___</v>
+        <v>Al técnico Víctor Manuel Vucetich le dicen el Rey ___</v>
       </c>
       <c r="D201" t="str">
-        <v>CAMPO</v>
+        <v>MIDAS</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B202" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C202" t="str">
-        <v>¿Cuántos jugadores tiene cada equipo en la cancha?</v>
+        <v>Al delantero chileno Humberto Suazo le decían «___»</v>
       </c>
       <c r="D202" t="str">
-        <v>ONCE</v>
+        <v>CHUPETE</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>BORREGOS</v>
+        <v>RAYADOS</v>
       </c>
       <c r="B203" t="str">
         <v>PREGUNTA</v>
       </c>
       <c r="C203" t="str">
-        <v>¿En cuántas oportunidades hay que avanzar diez yardas?</v>
+        <v>El máximo goleador en la historia de Rayados es Rogelio Funes ___</v>
       </c>
       <c r="D203" t="str">
-        <v>CUATRO</v>
+        <v>MORI</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
+        <v>RAYADOS</v>
+      </c>
+      <c r="B204" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Al ídolo regiomontano Jesús Arellano le decían «El ___»</v>
+      </c>
+      <c r="D204" t="str">
+        <v>CABRITO</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>RAYADOS</v>
+      </c>
+      <c r="B205" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C205" t="str">
+        <v>En 2025 llegó a Rayados el famoso defensa español Sergio ___</v>
+      </c>
+      <c r="D205" t="str">
+        <v>RAMOS</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>RAYADOS</v>
+      </c>
+      <c r="B206" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Rayados quedó en tercer lugar del Mundial de ___ en 2012 y en 2019</v>
+      </c>
+      <c r="D206" t="str">
+        <v>CLUBES</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>RAYADOS</v>
+      </c>
+      <c r="B207" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C207" t="str">
+        <v>A la barra de Rayados se le conoce como La ___</v>
+      </c>
+      <c r="D207" t="str">
+        <v>ADICCIÓN</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>RAYADOS</v>
+      </c>
+      <c r="B208" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C208" t="str">
+        <v>El partido entre Rayados y Tigres se llama el Clásico ___</v>
+      </c>
+      <c r="D208" t="str">
+        <v>REGIO</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>RAYADOS</v>
+      </c>
+      <c r="B209" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Monterrey es la capital del estado de Nuevo ___</v>
+      </c>
+      <c r="D209" t="str">
+        <v>LEÓN</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
         <v>BORREGOS</v>
       </c>
-      <c r="B204" t="str">
-        <v>PREGUNTA</v>
-      </c>
-      <c r="C204" t="str">
+      <c r="B210" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C210" t="str">
+        <v>El equipo del Tec de Monterrey se llama Borregos ___</v>
+      </c>
+      <c r="D210" t="str">
+        <v>SALVAJES</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B211" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Los Borregos juegan futbol ___</v>
+      </c>
+      <c r="D211" t="str">
+        <v>AMERICANO</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B212" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C212" t="str">
+        <v>Borregos es el equipo del Tecnológico de ___</v>
+      </c>
+      <c r="D212" t="str">
+        <v>MONTERREY</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B213" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C213" t="str">
+        <v>El Tec de Monterrey lo fundó el empresario Eugenio Garza ___</v>
+      </c>
+      <c r="D213" t="str">
+        <v>SADA</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B214" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C214" t="str">
+        <v>¿En qué año se fundó el Tec de Monterrey?</v>
+      </c>
+      <c r="D214" t="str">
+        <v>1943</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B215" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Los colores de Borregos son el azul y el ___</v>
+      </c>
+      <c r="D215" t="str">
+        <v>BLANCO</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B216" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C216" t="str">
+        <v>¿En qué año se inauguró el Estadio Borregos?</v>
+      </c>
+      <c r="D216" t="str">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B217" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C217" t="str">
+        <v>El Estadio Borregos se construyó en el lugar del antiguo Estadio ___</v>
+      </c>
+      <c r="D217" t="str">
+        <v>TECNOLÓGICO</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B218" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C218" t="str">
+        <v>¿Qué equipo de futbol soccer jugó en el Estadio Tecnológico hasta 2015?</v>
+      </c>
+      <c r="D218" t="str">
+        <v>RAYADOS</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B219" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C219" t="str">
+        <v>¿Cómo se llama la liga universitaria de futbol americano donde juega Borregos?</v>
+      </c>
+      <c r="D219" t="str">
+        <v>ONEFA</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B220" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C220" t="str">
+        <v>El gran rival universitario de Borregos son los Auténticos ___</v>
+      </c>
+      <c r="D220" t="str">
+        <v>TIGRES</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B221" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C221" t="str">
+        <v>El legendario coach de Borregos Monterrey fue Frank ___</v>
+      </c>
+      <c r="D221" t="str">
+        <v>GONZÁLEZ</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B222" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C222" t="str">
+        <v>¿Qué animal es la mascota del Tec de Monterrey?</v>
+      </c>
+      <c r="D222" t="str">
+        <v>BORREGO</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B223" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C223" t="str">
+        <v>Llevar el balón hasta la zona de anotación es un ___</v>
+      </c>
+      <c r="D223" t="str">
+        <v>TOUCHDOWN</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B224" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C224" t="str">
+        <v>¿Cuántos puntos vale un touchdown?</v>
+      </c>
+      <c r="D224" t="str">
+        <v>SEIS</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B225" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C225" t="str">
+        <v>¿Cuántos puntos vale un gol de campo?</v>
+      </c>
+      <c r="D225" t="str">
+        <v>TRES</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B226" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C226" t="str">
+        <v>¿Cuántos puntos vale un safety?</v>
+      </c>
+      <c r="D226" t="str">
+        <v>DOS</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B227" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C227" t="str">
+        <v>Después de un touchdown se patea para ganar el punto ___</v>
+      </c>
+      <c r="D227" t="str">
+        <v>EXTRA</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B228" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C228" t="str">
+        <v>El jugador que lanza los pases es el mariscal de ___</v>
+      </c>
+      <c r="D228" t="str">
+        <v>CAMPO</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B229" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C229" t="str">
+        <v>¿Cuántos jugadores tiene cada equipo en la cancha?</v>
+      </c>
+      <c r="D229" t="str">
+        <v>ONCE</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B230" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C230" t="str">
+        <v>¿En cuántas oportunidades hay que avanzar diez yardas?</v>
+      </c>
+      <c r="D230" t="str">
+        <v>CUATRO</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>BORREGOS</v>
+      </c>
+      <c r="B231" t="str">
+        <v>PREGUNTA</v>
+      </c>
+      <c r="C231" t="str">
         <v>La gran final de la NFL se llama el Super ___</v>
       </c>
-      <c r="D204" t="str">
+      <c r="D231" t="str">
         <v>BOWL</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D204"/>
+  <autoFilter ref="A1:D231"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D204"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D231"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>